<commit_message>
Tim bai theo ma tren URL de panel mo duoc tren moi giao dien Threads
- Khong lay bai goc co dinh o threads_post_page_0 (co ban Threads de rong)
- Mo link cua mot comment: tra loi dung comment do, gui kem bai cha lam ngu canh
- Nhan o soan cua bai goc theo username, khong phu thuoc chu "Reply to"
- Cap nhat data/seeding.xlsx

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01V2rL2vCuk9fzvm3RthQJ4r
</commit_message>
<xml_diff>
--- a/data/seeding.xlsx
+++ b/data/seeding.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Seeding-media\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\freelancer\baotran\affliate-comment\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97ABC56D-5872-4CA5-BF7F-51528A6CB5CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E919DBF-FD03-4FDB-8676-A43EC8B2B593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{FB351C2D-D222-4FD7-8A1F-0AFAF061EB0D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FB351C2D-D222-4FD7-8A1F-0AFAF061EB0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Chăm sóc da mặt - body " sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="615" uniqueCount="604">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="608">
   <si>
     <t>Link rút gọn - CHĂM SÓC DA</t>
   </si>
@@ -1863,6 +1863,18 @@
   </si>
   <si>
     <t>Combo 1kg Bánh Tráng Rìa Ủ Bơ Muối Ghiền Hành Phi Sốt Tắc</t>
+  </si>
+  <si>
+    <t>Mô tả</t>
+  </si>
+  <si>
+    <t>Giá</t>
+  </si>
+  <si>
+    <t>mô tả</t>
+  </si>
+  <si>
+    <t>giá</t>
   </si>
 </sst>
 </file>
@@ -2017,9 +2029,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2040,6 +2049,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2376,24 +2388,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A76331EE-B366-4432-B230-84D3FD36ABDD}">
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" customWidth="1"/>
     <col min="2" max="2" width="44" style="13" customWidth="1"/>
-    <col min="3" max="3" width="52.44140625" style="15" customWidth="1"/>
-    <col min="4" max="4" width="29.77734375" customWidth="1"/>
+    <col min="3" max="5" width="52.44140625" style="15" customWidth="1"/>
+    <col min="6" max="6" width="29.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -2404,10 +2418,16 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>606</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>607</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -2417,9 +2437,11 @@
       <c r="C3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -2429,9 +2451,11 @@
       <c r="C4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -2441,9 +2465,11 @@
       <c r="C5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="6"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -2453,9 +2479,11 @@
       <c r="C6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -2465,9 +2493,11 @@
       <c r="C7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -2477,9 +2507,11 @@
       <c r="C8" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -2489,9 +2521,11 @@
       <c r="C9" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -2501,9 +2535,11 @@
       <c r="C10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -2513,9 +2549,11 @@
       <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="6"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -2525,9 +2563,11 @@
       <c r="C12" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -2537,9 +2577,11 @@
       <c r="C13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -2549,9 +2591,11 @@
       <c r="C14" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -2561,9 +2605,11 @@
       <c r="C15" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -2573,9 +2619,11 @@
       <c r="C16" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -2585,9 +2633,11 @@
       <c r="C17" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -2597,9 +2647,11 @@
       <c r="C18" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -2609,9 +2661,11 @@
       <c r="C19" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -2621,9 +2675,11 @@
       <c r="C20" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -2633,9 +2689,11 @@
       <c r="C21" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -2645,9 +2703,11 @@
       <c r="C22" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>21</v>
       </c>
@@ -2657,9 +2717,11 @@
       <c r="C23" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>22</v>
       </c>
@@ -2669,9 +2731,11 @@
       <c r="C24" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>23</v>
       </c>
@@ -2681,9 +2745,11 @@
       <c r="C25" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -2693,9 +2759,11 @@
       <c r="C26" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="6"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -2705,9 +2773,11 @@
       <c r="C27" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="6"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -2717,9 +2787,11 @@
       <c r="C28" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="D28" s="6"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -2729,9 +2801,11 @@
       <c r="C29" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="D29" s="6"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -2741,9 +2815,11 @@
       <c r="C30" s="10" t="s">
         <v>67</v>
       </c>
-      <c r="D30" s="6"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -2753,9 +2829,11 @@
       <c r="C31" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="D31" s="6"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -2765,9 +2843,11 @@
       <c r="C32" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="D32" s="6"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>31</v>
       </c>
@@ -2777,9 +2857,11 @@
       <c r="C33" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="D33" s="6"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>32</v>
       </c>
@@ -2789,9 +2871,11 @@
       <c r="C34" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="D34" s="6"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>33</v>
       </c>
@@ -2801,9 +2885,11 @@
       <c r="C35" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="D35" s="6"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>34</v>
       </c>
@@ -2813,9 +2899,11 @@
       <c r="C36" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D36" s="6"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="6"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>35</v>
       </c>
@@ -2825,9 +2913,11 @@
       <c r="C37" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="D37" s="6"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="6"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>36</v>
       </c>
@@ -2837,9 +2927,11 @@
       <c r="C38" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="D38" s="6"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="6"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>37</v>
       </c>
@@ -2849,9 +2941,11 @@
       <c r="C39" s="10" t="s">
         <v>85</v>
       </c>
-      <c r="D39" s="6"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>38</v>
       </c>
@@ -2861,9 +2955,11 @@
       <c r="C40" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="D40" s="6"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="6"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>39</v>
       </c>
@@ -2873,9 +2969,11 @@
       <c r="C41" s="10" t="s">
         <v>89</v>
       </c>
-      <c r="D41" s="6"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="6"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>40</v>
       </c>
@@ -2885,9 +2983,11 @@
       <c r="C42" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="D42" s="6"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="6"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>41</v>
       </c>
@@ -2897,9 +2997,11 @@
       <c r="C43" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="6"/>
+    </row>
+    <row r="44" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>42</v>
       </c>
@@ -2909,9 +3011,11 @@
       <c r="C44" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="6"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>43</v>
       </c>
@@ -2921,9 +3025,11 @@
       <c r="C45" s="10" t="s">
         <v>97</v>
       </c>
-      <c r="D45" s="6"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="6"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>44</v>
       </c>
@@ -2933,9 +3039,11 @@
       <c r="C46" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="D46" s="6"/>
-    </row>
-    <row r="47" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="6"/>
+    </row>
+    <row r="47" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>45</v>
       </c>
@@ -2945,9 +3053,11 @@
       <c r="C47" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="D47" s="6"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="6"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
         <v>46</v>
       </c>
@@ -2957,9 +3067,11 @@
       <c r="C48" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="6"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>47</v>
       </c>
@@ -2969,9 +3081,11 @@
       <c r="C49" s="10" t="s">
         <v>105</v>
       </c>
-      <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="6"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>48</v>
       </c>
@@ -2981,9 +3095,11 @@
       <c r="C50" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="D50" s="6"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="6"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>49</v>
       </c>
@@ -2993,9 +3109,11 @@
       <c r="C51" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="6"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>50</v>
       </c>
@@ -3005,9 +3123,11 @@
       <c r="C52" s="10" t="s">
         <v>111</v>
       </c>
-      <c r="D52" s="6"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="6"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>51</v>
       </c>
@@ -3017,9 +3137,11 @@
       <c r="C53" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="D53" s="6"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="6"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>52</v>
       </c>
@@ -3029,9 +3151,11 @@
       <c r="C54" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="6"/>
+    </row>
+    <row r="55" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>53</v>
       </c>
@@ -3041,9 +3165,11 @@
       <c r="C55" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="D55" s="6"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="6"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>54</v>
       </c>
@@ -3053,9 +3179,11 @@
       <c r="C56" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="D56" s="6"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D56" s="10"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="6"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>55</v>
       </c>
@@ -3065,9 +3193,11 @@
       <c r="C57" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="D57" s="7"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>56</v>
       </c>
@@ -3077,9 +3207,11 @@
       <c r="C58" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="D58" s="7"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>57</v>
       </c>
@@ -3089,9 +3221,11 @@
       <c r="C59" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="D59" s="7"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>58</v>
       </c>
@@ -3101,9 +3235,11 @@
       <c r="C60" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="D60" s="7"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="7"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>59</v>
       </c>
@@ -3113,9 +3249,11 @@
       <c r="C61" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D61" s="7"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="7"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="3">
         <v>60</v>
       </c>
@@ -3125,9 +3263,11 @@
       <c r="C62" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="D62" s="7"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="3">
         <v>61</v>
       </c>
@@ -3137,9 +3277,11 @@
       <c r="C63" s="5" t="s">
         <v>133</v>
       </c>
-      <c r="D63" s="7"/>
-    </row>
-    <row r="64" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="7"/>
+    </row>
+    <row r="64" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A64" s="3">
         <v>62</v>
       </c>
@@ -3149,9 +3291,11 @@
       <c r="C64" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D64" s="7"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="7"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="3">
         <v>63</v>
       </c>
@@ -3161,9 +3305,11 @@
       <c r="C65" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="D65" s="7"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="7"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="3">
         <v>64</v>
       </c>
@@ -3173,9 +3319,11 @@
       <c r="C66" s="5" t="s">
         <v>139</v>
       </c>
-      <c r="D66" s="7"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="7"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="3">
         <v>65</v>
       </c>
@@ -3185,9 +3333,11 @@
       <c r="C67" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="D67" s="7"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="7"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="3">
         <v>66</v>
       </c>
@@ -3197,9 +3347,11 @@
       <c r="C68" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="D68" s="7"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="7"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="3">
         <v>67</v>
       </c>
@@ -3209,9 +3361,11 @@
       <c r="C69" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="D69" s="7"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="7"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="3">
         <v>68</v>
       </c>
@@ -3221,9 +3375,11 @@
       <c r="C70" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D70" s="7"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="3">
         <v>69</v>
       </c>
@@ -3233,9 +3389,11 @@
       <c r="C71" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="D71" s="7"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="7"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="3">
         <v>70</v>
       </c>
@@ -3245,9 +3403,11 @@
       <c r="C72" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="D72" s="7"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="3">
         <v>71</v>
       </c>
@@ -3257,9 +3417,11 @@
       <c r="C73" s="14" t="s">
         <v>153</v>
       </c>
-      <c r="D73" s="1"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D73" s="14"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="1"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="3">
         <v>72</v>
       </c>
@@ -3269,9 +3431,11 @@
       <c r="C74" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="D74" s="1"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D74" s="14"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="1"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="3">
         <v>73</v>
       </c>
@@ -3281,9 +3445,11 @@
       <c r="C75" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="D75" s="1"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="1"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="3">
         <v>74</v>
       </c>
@@ -3293,9 +3459,11 @@
       <c r="C76" s="14" t="s">
         <v>159</v>
       </c>
-      <c r="D76" s="1"/>
-    </row>
-    <row r="77" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="1"/>
+    </row>
+    <row r="77" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A77" s="3">
         <v>75</v>
       </c>
@@ -3305,9 +3473,11 @@
       <c r="C77" s="14" t="s">
         <v>161</v>
       </c>
-      <c r="D77" s="1"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="1"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="3">
         <v>76</v>
       </c>
@@ -3317,9 +3487,11 @@
       <c r="C78" s="14" t="s">
         <v>163</v>
       </c>
-      <c r="D78" s="1"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D78" s="14"/>
+      <c r="E78" s="14"/>
+      <c r="F78" s="1"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="3">
         <v>77</v>
       </c>
@@ -3329,9 +3501,11 @@
       <c r="C79" s="14" t="s">
         <v>165</v>
       </c>
-      <c r="D79" s="1"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D79" s="14"/>
+      <c r="E79" s="14"/>
+      <c r="F79" s="1"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="3">
         <v>78</v>
       </c>
@@ -3341,9 +3515,11 @@
       <c r="C80" s="14" t="s">
         <v>166</v>
       </c>
-      <c r="D80" s="1"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D80" s="14"/>
+      <c r="E80" s="14"/>
+      <c r="F80" s="1"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="3">
         <v>79</v>
       </c>
@@ -3353,9 +3529,11 @@
       <c r="C81" s="14" t="s">
         <v>167</v>
       </c>
-      <c r="D81" s="1"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D81" s="14"/>
+      <c r="E81" s="14"/>
+      <c r="F81" s="1"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="3">
         <v>80</v>
       </c>
@@ -3365,9 +3543,11 @@
       <c r="C82" s="14" t="s">
         <v>170</v>
       </c>
-      <c r="D82" s="1"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D82" s="14"/>
+      <c r="E82" s="14"/>
+      <c r="F82" s="1"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="3">
         <v>81</v>
       </c>
@@ -3377,9 +3557,11 @@
       <c r="C83" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="D83" s="1"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D83" s="14"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="1"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="3">
         <v>82</v>
       </c>
@@ -3389,9 +3571,11 @@
       <c r="C84" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="D84" s="1"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D84" s="14"/>
+      <c r="E84" s="14"/>
+      <c r="F84" s="1"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="3">
         <v>83</v>
       </c>
@@ -3401,9 +3585,11 @@
       <c r="C85" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="D85" s="1"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D85" s="14"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="1"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="3">
         <v>84</v>
       </c>
@@ -3413,9 +3599,11 @@
       <c r="C86" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="D86" s="1"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D86" s="14"/>
+      <c r="E86" s="14"/>
+      <c r="F86" s="1"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="3">
         <v>85</v>
       </c>
@@ -3425,9 +3613,11 @@
       <c r="C87" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="D87" s="1"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D87" s="14"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="1"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="3">
         <v>86</v>
       </c>
@@ -3437,9 +3627,11 @@
       <c r="C88" s="14" t="s">
         <v>182</v>
       </c>
-      <c r="D88" s="1"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D88" s="14"/>
+      <c r="E88" s="14"/>
+      <c r="F88" s="1"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="3">
         <v>87</v>
       </c>
@@ -3449,9 +3641,11 @@
       <c r="C89" s="14" t="s">
         <v>184</v>
       </c>
-      <c r="D89" s="1"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D89" s="14"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="1"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="3">
         <v>88</v>
       </c>
@@ -3461,9 +3655,11 @@
       <c r="C90" s="14" t="s">
         <v>186</v>
       </c>
-      <c r="D90" s="1"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D90" s="14"/>
+      <c r="E90" s="14"/>
+      <c r="F90" s="1"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="3">
         <v>89</v>
       </c>
@@ -3473,9 +3669,11 @@
       <c r="C91" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="D91" s="1"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D91" s="14"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="1"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="3">
         <v>90</v>
       </c>
@@ -3485,9 +3683,11 @@
       <c r="C92" s="14" t="s">
         <v>190</v>
       </c>
-      <c r="D92" s="1"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D92" s="14"/>
+      <c r="E92" s="14"/>
+      <c r="F92" s="1"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="3">
         <v>91</v>
       </c>
@@ -3497,9 +3697,11 @@
       <c r="C93" s="14" t="s">
         <v>192</v>
       </c>
-      <c r="D93" s="1"/>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D93" s="14"/>
+      <c r="E93" s="14"/>
+      <c r="F93" s="1"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="3">
         <v>92</v>
       </c>
@@ -3509,9 +3711,11 @@
       <c r="C94" s="14" t="s">
         <v>194</v>
       </c>
-      <c r="D94" s="1"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D94" s="14"/>
+      <c r="E94" s="14"/>
+      <c r="F94" s="1"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="3">
         <v>93</v>
       </c>
@@ -3521,9 +3725,11 @@
       <c r="C95" s="14" t="s">
         <v>196</v>
       </c>
-      <c r="D95" s="1"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D95" s="14"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="1"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="3">
         <v>94</v>
       </c>
@@ -3533,9 +3739,11 @@
       <c r="C96" s="14" t="s">
         <v>198</v>
       </c>
-      <c r="D96" s="1"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D96" s="14"/>
+      <c r="E96" s="14"/>
+      <c r="F96" s="1"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="3">
         <v>95</v>
       </c>
@@ -3545,9 +3753,11 @@
       <c r="C97" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="D97" s="1"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D97" s="14"/>
+      <c r="E97" s="14"/>
+      <c r="F97" s="1"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="3">
         <v>96</v>
       </c>
@@ -3557,9 +3767,11 @@
       <c r="C98" s="14" t="s">
         <v>202</v>
       </c>
-      <c r="D98" s="1"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D98" s="14"/>
+      <c r="E98" s="14"/>
+      <c r="F98" s="1"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="3">
         <v>97</v>
       </c>
@@ -3569,9 +3781,11 @@
       <c r="C99" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="D99" s="1"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D99" s="14"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="1"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="3">
         <v>98</v>
       </c>
@@ -3581,9 +3795,11 @@
       <c r="C100" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="D100" s="1"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D100" s="14"/>
+      <c r="E100" s="14"/>
+      <c r="F100" s="1"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="3">
         <v>99</v>
       </c>
@@ -3593,9 +3809,11 @@
       <c r="C101" s="14" t="s">
         <v>208</v>
       </c>
-      <c r="D101" s="1"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D101" s="14"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="1"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="3">
         <v>100</v>
       </c>
@@ -3605,11 +3823,13 @@
       <c r="C102" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="D102" s="1"/>
+      <c r="D102" s="14"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{383E355E-1B99-430B-9806-D857BD3E2B13}"/>
@@ -3719,24 +3939,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0F58A854-B478-4E6C-BF65-3003D1F2AB36}">
-  <dimension ref="A1:D102"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.5546875" customWidth="1"/>
-    <col min="2" max="2" width="35.5546875" style="21" customWidth="1"/>
-    <col min="3" max="3" width="35.6640625" style="15" customWidth="1"/>
-    <col min="4" max="4" width="18.88671875" customWidth="1"/>
+    <col min="2" max="2" width="35.5546875" style="20" customWidth="1"/>
+    <col min="3" max="5" width="35.6640625" style="15" customWidth="1"/>
+    <col min="6" max="6" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6" ht="19.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -3747,22 +3969,30 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3772,9 +4002,11 @@
       <c r="C4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5" spans="1:4" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" spans="1:6" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3784,9 +4016,11 @@
       <c r="C5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="6"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3796,9 +4030,11 @@
       <c r="C6" s="5" t="s">
         <v>212</v>
       </c>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3808,9 +4044,11 @@
       <c r="C7" s="5" t="s">
         <v>213</v>
       </c>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D7" s="5"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3820,9 +4058,11 @@
       <c r="C8" s="5" t="s">
         <v>216</v>
       </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3832,9 +4072,11 @@
       <c r="C9" s="5" t="s">
         <v>218</v>
       </c>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3844,9 +4086,11 @@
       <c r="C10" s="5" t="s">
         <v>219</v>
       </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
+      <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3856,9 +4100,11 @@
       <c r="C11" s="5" t="s">
         <v>222</v>
       </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="6"/>
+    </row>
+    <row r="12" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3868,9 +4114,11 @@
       <c r="C12" s="5" t="s">
         <v>224</v>
       </c>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3880,9 +4128,11 @@
       <c r="C13" s="5" t="s">
         <v>226</v>
       </c>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D13" s="5"/>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3892,9 +4142,11 @@
       <c r="C14" s="5" t="s">
         <v>228</v>
       </c>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -3904,9 +4156,11 @@
       <c r="C15" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:4" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -3916,9 +4170,11 @@
       <c r="C16" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -3928,9 +4184,11 @@
       <c r="C17" s="10" t="s">
         <v>234</v>
       </c>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -3940,9 +4198,11 @@
       <c r="C18" s="10" t="s">
         <v>236</v>
       </c>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -3952,9 +4212,11 @@
       <c r="C19" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -3964,9 +4226,11 @@
       <c r="C20" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -3976,9 +4240,11 @@
       <c r="C21" s="10" t="s">
         <v>242</v>
       </c>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -3988,9 +4254,11 @@
       <c r="C22" s="10" t="s">
         <v>244</v>
       </c>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D22" s="10"/>
+      <c r="E22" s="10"/>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>21</v>
       </c>
@@ -4000,9 +4268,11 @@
       <c r="C23" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D23" s="10"/>
+      <c r="E23" s="10"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>22</v>
       </c>
@@ -4012,9 +4282,11 @@
       <c r="C24" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>23</v>
       </c>
@@ -4024,9 +4296,11 @@
       <c r="C25" s="10" t="s">
         <v>250</v>
       </c>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -4036,9 +4310,11 @@
       <c r="C26" s="10" t="s">
         <v>252</v>
       </c>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="6"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -4048,9 +4324,11 @@
       <c r="C27" s="10" t="s">
         <v>254</v>
       </c>
-      <c r="D27" s="6"/>
-    </row>
-    <row r="28" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D27" s="10"/>
+      <c r="E27" s="10"/>
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -4060,9 +4338,11 @@
       <c r="C28" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="D28" s="6"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D28" s="10"/>
+      <c r="E28" s="10"/>
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -4072,9 +4352,11 @@
       <c r="C29" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="D29" s="6"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -4084,9 +4366,11 @@
       <c r="C30" s="10" t="s">
         <v>260</v>
       </c>
-      <c r="D30" s="6"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D30" s="10"/>
+      <c r="E30" s="10"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -4096,9 +4380,11 @@
       <c r="C31" s="10" t="s">
         <v>262</v>
       </c>
-      <c r="D31" s="6"/>
-    </row>
-    <row r="32" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -4108,9 +4394,11 @@
       <c r="C32" s="10" t="s">
         <v>264</v>
       </c>
-      <c r="D32" s="6"/>
-    </row>
-    <row r="33" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>31</v>
       </c>
@@ -4120,9 +4408,11 @@
       <c r="C33" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="D33" s="6"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>32</v>
       </c>
@@ -4132,9 +4422,11 @@
       <c r="C34" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="D34" s="6"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>33</v>
       </c>
@@ -4144,9 +4436,11 @@
       <c r="C35" s="10" t="s">
         <v>269</v>
       </c>
-      <c r="D35" s="6"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>34</v>
       </c>
@@ -4156,9 +4450,11 @@
       <c r="C36" s="10" t="s">
         <v>272</v>
       </c>
-      <c r="D36" s="6"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="6"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>35</v>
       </c>
@@ -4168,9 +4464,11 @@
       <c r="C37" s="10" t="s">
         <v>274</v>
       </c>
-      <c r="D37" s="6"/>
-    </row>
-    <row r="38" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="6"/>
+    </row>
+    <row r="38" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>36</v>
       </c>
@@ -4180,9 +4478,11 @@
       <c r="C38" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="D38" s="6"/>
-    </row>
-    <row r="39" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="6"/>
+    </row>
+    <row r="39" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>37</v>
       </c>
@@ -4192,9 +4492,11 @@
       <c r="C39" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="D39" s="6"/>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>38</v>
       </c>
@@ -4204,21 +4506,25 @@
       <c r="C40" s="10" t="s">
         <v>280</v>
       </c>
-      <c r="D40" s="6"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="6"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>39</v>
       </c>
-      <c r="B41" s="19" t="s">
+      <c r="B41" s="18" t="s">
         <v>281</v>
       </c>
       <c r="C41" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="D41" s="6"/>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="6"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>40</v>
       </c>
@@ -4228,9 +4534,11 @@
       <c r="C42" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="D42" s="6"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="6"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>41</v>
       </c>
@@ -4240,9 +4548,11 @@
       <c r="C43" s="10" t="s">
         <v>286</v>
       </c>
-      <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="6"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>42</v>
       </c>
@@ -4252,9 +4562,11 @@
       <c r="C44" s="10" t="s">
         <v>288</v>
       </c>
-      <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="6"/>
+    </row>
+    <row r="45" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>43</v>
       </c>
@@ -4264,9 +4576,11 @@
       <c r="C45" s="10" t="s">
         <v>289</v>
       </c>
-      <c r="D45" s="6"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="6"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>44</v>
       </c>
@@ -4276,9 +4590,11 @@
       <c r="C46" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="D46" s="6"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="6"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>45</v>
       </c>
@@ -4288,9 +4604,11 @@
       <c r="C47" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="D47" s="6"/>
-    </row>
-    <row r="48" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="6"/>
+    </row>
+    <row r="48" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
         <v>46</v>
       </c>
@@ -4300,9 +4618,11 @@
       <c r="C48" s="10" t="s">
         <v>295</v>
       </c>
-      <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="6"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>47</v>
       </c>
@@ -4312,9 +4632,11 @@
       <c r="C49" s="10" t="s">
         <v>297</v>
       </c>
-      <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="6"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>48</v>
       </c>
@@ -4324,9 +4646,11 @@
       <c r="C50" s="10" t="s">
         <v>299</v>
       </c>
-      <c r="D50" s="6"/>
-    </row>
-    <row r="51" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="6"/>
+    </row>
+    <row r="51" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>49</v>
       </c>
@@ -4336,9 +4660,11 @@
       <c r="C51" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="6"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>50</v>
       </c>
@@ -4348,9 +4674,11 @@
       <c r="C52" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D52" s="6"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="6"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>51</v>
       </c>
@@ -4360,9 +4688,11 @@
       <c r="C53" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="D53" s="6"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="6"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>52</v>
       </c>
@@ -4372,9 +4702,11 @@
       <c r="C54" s="10" t="s">
         <v>306</v>
       </c>
-      <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="6"/>
+    </row>
+    <row r="55" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>53</v>
       </c>
@@ -4384,9 +4716,11 @@
       <c r="C55" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="D55" s="6"/>
-    </row>
-    <row r="56" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="6"/>
+    </row>
+    <row r="56" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>54</v>
       </c>
@@ -4396,9 +4730,11 @@
       <c r="C56" s="10" t="s">
         <v>311</v>
       </c>
-      <c r="D56" s="6"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D56" s="10"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="6"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>55</v>
       </c>
@@ -4408,9 +4744,11 @@
       <c r="C57" s="5" t="s">
         <v>312</v>
       </c>
-      <c r="D57" s="7"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>56</v>
       </c>
@@ -4420,9 +4758,11 @@
       <c r="C58" s="5" t="s">
         <v>315</v>
       </c>
-      <c r="D58" s="7"/>
-    </row>
-    <row r="59" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>57</v>
       </c>
@@ -4432,9 +4772,11 @@
       <c r="C59" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="D59" s="7"/>
-    </row>
-    <row r="60" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>58</v>
       </c>
@@ -4444,9 +4786,11 @@
       <c r="C60" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="D60" s="7"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="7"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>59</v>
       </c>
@@ -4456,9 +4800,11 @@
       <c r="C61" s="5" t="s">
         <v>321</v>
       </c>
-      <c r="D61" s="7"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="7"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="3">
         <v>60</v>
       </c>
@@ -4468,9 +4814,11 @@
       <c r="C62" s="5" t="s">
         <v>323</v>
       </c>
-      <c r="D62" s="7"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="3">
         <v>61</v>
       </c>
@@ -4480,9 +4828,11 @@
       <c r="C63" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="D63" s="7"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="7"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="3">
         <v>62</v>
       </c>
@@ -4492,9 +4842,11 @@
       <c r="C64" s="5" t="s">
         <v>327</v>
       </c>
-      <c r="D64" s="7"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="7"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="3">
         <v>63</v>
       </c>
@@ -4504,9 +4856,11 @@
       <c r="C65" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="D65" s="7"/>
-    </row>
-    <row r="66" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="7"/>
+    </row>
+    <row r="66" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A66" s="3">
         <v>64</v>
       </c>
@@ -4516,9 +4870,11 @@
       <c r="C66" s="5" t="s">
         <v>331</v>
       </c>
-      <c r="D66" s="7"/>
-    </row>
-    <row r="67" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="7"/>
+    </row>
+    <row r="67" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A67" s="3">
         <v>65</v>
       </c>
@@ -4528,9 +4884,11 @@
       <c r="C67" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="D67" s="7"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="7"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="3">
         <v>66</v>
       </c>
@@ -4540,9 +4898,11 @@
       <c r="C68" s="5" t="s">
         <v>335</v>
       </c>
-      <c r="D68" s="7"/>
-    </row>
-    <row r="69" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="7"/>
+    </row>
+    <row r="69" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A69" s="3">
         <v>67</v>
       </c>
@@ -4552,9 +4912,11 @@
       <c r="C69" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="D69" s="7"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="7"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="3">
         <v>68</v>
       </c>
@@ -4564,9 +4926,11 @@
       <c r="C70" s="5" t="s">
         <v>339</v>
       </c>
-      <c r="D70" s="7"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="3">
         <v>69</v>
       </c>
@@ -4576,9 +4940,11 @@
       <c r="C71" s="5" t="s">
         <v>341</v>
       </c>
-      <c r="D71" s="7"/>
-    </row>
-    <row r="72" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="7"/>
+    </row>
+    <row r="72" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A72" s="3">
         <v>70</v>
       </c>
@@ -4588,371 +4954,433 @@
       <c r="C72" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="D72" s="7"/>
-    </row>
-    <row r="73" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A73" s="3">
         <v>71</v>
       </c>
-      <c r="B73" s="20" t="s">
+      <c r="B73" s="19" t="s">
         <v>344</v>
       </c>
       <c r="C73" s="14" t="s">
         <v>345</v>
       </c>
-      <c r="D73" s="1"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D73" s="14"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="1"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="3">
         <v>72</v>
       </c>
-      <c r="B74" s="20" t="s">
+      <c r="B74" s="19" t="s">
         <v>346</v>
       </c>
       <c r="C74" s="14" t="s">
         <v>347</v>
       </c>
-      <c r="D74" s="1"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D74" s="14"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="1"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="3">
         <v>73</v>
       </c>
-      <c r="B75" s="20" t="s">
+      <c r="B75" s="19" t="s">
         <v>348</v>
       </c>
       <c r="C75" s="14" t="s">
         <v>349</v>
       </c>
-      <c r="D75" s="1"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="1"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="3">
         <v>74</v>
       </c>
-      <c r="B76" s="20" t="s">
+      <c r="B76" s="19" t="s">
         <v>350</v>
       </c>
       <c r="C76" s="14" t="s">
         <v>351</v>
       </c>
-      <c r="D76" s="1"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="1"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="3">
         <v>75</v>
       </c>
-      <c r="B77" s="20" t="s">
+      <c r="B77" s="19" t="s">
         <v>352</v>
       </c>
       <c r="C77" s="14" t="s">
         <v>353</v>
       </c>
-      <c r="D77" s="1"/>
-    </row>
-    <row r="78" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="1"/>
+    </row>
+    <row r="78" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A78" s="3">
         <v>76</v>
       </c>
-      <c r="B78" s="20" t="s">
+      <c r="B78" s="19" t="s">
         <v>354</v>
       </c>
       <c r="C78" s="14" t="s">
         <v>355</v>
       </c>
-      <c r="D78" s="1"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D78" s="14"/>
+      <c r="E78" s="14"/>
+      <c r="F78" s="1"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="3">
         <v>77</v>
       </c>
-      <c r="B79" s="20" t="s">
+      <c r="B79" s="19" t="s">
         <v>356</v>
       </c>
       <c r="C79" s="14" t="s">
         <v>357</v>
       </c>
-      <c r="D79" s="1"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D79" s="14"/>
+      <c r="E79" s="14"/>
+      <c r="F79" s="1"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="3">
         <v>78</v>
       </c>
-      <c r="B80" s="20" t="s">
+      <c r="B80" s="19" t="s">
         <v>358</v>
       </c>
       <c r="C80" s="14" t="s">
         <v>359</v>
       </c>
-      <c r="D80" s="1"/>
-    </row>
-    <row r="81" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D80" s="14"/>
+      <c r="E80" s="14"/>
+      <c r="F80" s="1"/>
+    </row>
+    <row r="81" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A81" s="3">
         <v>79</v>
       </c>
-      <c r="B81" s="20" t="s">
+      <c r="B81" s="19" t="s">
         <v>360</v>
       </c>
       <c r="C81" s="14" t="s">
         <v>361</v>
       </c>
-      <c r="D81" s="1"/>
-    </row>
-    <row r="82" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D81" s="14"/>
+      <c r="E81" s="14"/>
+      <c r="F81" s="1"/>
+    </row>
+    <row r="82" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A82" s="3">
         <v>80</v>
       </c>
-      <c r="B82" s="20" t="s">
+      <c r="B82" s="19" t="s">
         <v>362</v>
       </c>
       <c r="C82" s="14" t="s">
         <v>363</v>
       </c>
-      <c r="D82" s="1"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D82" s="14"/>
+      <c r="E82" s="14"/>
+      <c r="F82" s="1"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="3">
         <v>81</v>
       </c>
-      <c r="B83" s="20" t="s">
+      <c r="B83" s="19" t="s">
         <v>364</v>
       </c>
       <c r="C83" s="14" t="s">
         <v>365</v>
       </c>
-      <c r="D83" s="1"/>
-    </row>
-    <row r="84" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D83" s="14"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="1"/>
+    </row>
+    <row r="84" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A84" s="3">
         <v>82</v>
       </c>
-      <c r="B84" s="20" t="s">
+      <c r="B84" s="19" t="s">
         <v>366</v>
       </c>
       <c r="C84" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="D84" s="1"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D84" s="9"/>
+      <c r="E84" s="9"/>
+      <c r="F84" s="1"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="3">
         <v>83</v>
       </c>
-      <c r="B85" s="20" t="s">
+      <c r="B85" s="19" t="s">
         <v>368</v>
       </c>
       <c r="C85" s="14" t="s">
         <v>369</v>
       </c>
-      <c r="D85" s="1"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D85" s="14"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="1"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="3">
         <v>84</v>
       </c>
-      <c r="B86" s="20" t="s">
+      <c r="B86" s="19" t="s">
         <v>370</v>
       </c>
       <c r="C86" s="14" t="s">
         <v>371</v>
       </c>
-      <c r="D86" s="1"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D86" s="14"/>
+      <c r="E86" s="14"/>
+      <c r="F86" s="1"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="3">
         <v>85</v>
       </c>
-      <c r="B87" s="20" t="s">
+      <c r="B87" s="19" t="s">
         <v>374</v>
       </c>
       <c r="C87" s="14" t="s">
         <v>372</v>
       </c>
-      <c r="D87" s="1"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D87" s="14"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="1"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="3">
         <v>86</v>
       </c>
-      <c r="B88" s="20" t="s">
+      <c r="B88" s="19" t="s">
         <v>373</v>
       </c>
       <c r="C88" s="14" t="s">
         <v>375</v>
       </c>
-      <c r="D88" s="1"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D88" s="14"/>
+      <c r="E88" s="14"/>
+      <c r="F88" s="1"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="3">
         <v>87</v>
       </c>
-      <c r="B89" s="20" t="s">
+      <c r="B89" s="19" t="s">
         <v>376</v>
       </c>
       <c r="C89" s="14" t="s">
         <v>377</v>
       </c>
-      <c r="D89" s="1"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D89" s="14"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="1"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="3">
         <v>88</v>
       </c>
-      <c r="B90" s="20" t="s">
+      <c r="B90" s="19" t="s">
         <v>378</v>
       </c>
       <c r="C90" s="14" t="s">
         <v>379</v>
       </c>
-      <c r="D90" s="1"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D90" s="14"/>
+      <c r="E90" s="14"/>
+      <c r="F90" s="1"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="3">
         <v>89</v>
       </c>
-      <c r="B91" s="20" t="s">
+      <c r="B91" s="19" t="s">
         <v>380</v>
       </c>
       <c r="C91" s="14" t="s">
         <v>381</v>
       </c>
-      <c r="D91" s="1"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D91" s="14"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="1"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="3">
         <v>90</v>
       </c>
-      <c r="B92" s="20" t="s">
+      <c r="B92" s="19" t="s">
         <v>382</v>
       </c>
       <c r="C92" s="14" t="s">
         <v>383</v>
       </c>
-      <c r="D92" s="1"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D92" s="14"/>
+      <c r="E92" s="14"/>
+      <c r="F92" s="1"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="3">
         <v>91</v>
       </c>
-      <c r="B93" s="20" t="s">
+      <c r="B93" s="19" t="s">
         <v>384</v>
       </c>
       <c r="C93" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="D93" s="1"/>
-    </row>
-    <row r="94" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D93" s="14"/>
+      <c r="E93" s="14"/>
+      <c r="F93" s="1"/>
+    </row>
+    <row r="94" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A94" s="3">
         <v>92</v>
       </c>
-      <c r="B94" s="20" t="s">
+      <c r="B94" s="19" t="s">
         <v>386</v>
       </c>
       <c r="C94" s="14" t="s">
         <v>387</v>
       </c>
-      <c r="D94" s="1"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D94" s="14"/>
+      <c r="E94" s="14"/>
+      <c r="F94" s="1"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="3">
         <v>93</v>
       </c>
-      <c r="B95" s="20" t="s">
+      <c r="B95" s="19" t="s">
         <v>388</v>
       </c>
       <c r="C95" s="14" t="s">
         <v>389</v>
       </c>
-      <c r="D95" s="1"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D95" s="14"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="1"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="3">
         <v>94</v>
       </c>
-      <c r="B96" s="20" t="s">
+      <c r="B96" s="19" t="s">
         <v>390</v>
       </c>
       <c r="C96" s="14" t="s">
         <v>393</v>
       </c>
-      <c r="D96" s="1"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D96" s="14"/>
+      <c r="E96" s="14"/>
+      <c r="F96" s="1"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="3">
         <v>95</v>
       </c>
-      <c r="B97" s="20" t="s">
+      <c r="B97" s="19" t="s">
         <v>391</v>
       </c>
       <c r="C97" s="14" t="s">
         <v>392</v>
       </c>
-      <c r="D97" s="1"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D97" s="14"/>
+      <c r="E97" s="14"/>
+      <c r="F97" s="1"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="3">
         <v>96</v>
       </c>
-      <c r="B98" s="20" t="s">
+      <c r="B98" s="19" t="s">
         <v>394</v>
       </c>
       <c r="C98" s="14" t="s">
         <v>395</v>
       </c>
-      <c r="D98" s="1"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D98" s="14"/>
+      <c r="E98" s="14"/>
+      <c r="F98" s="1"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="3">
         <v>97</v>
       </c>
-      <c r="B99" s="20" t="s">
+      <c r="B99" s="19" t="s">
         <v>396</v>
       </c>
       <c r="C99" s="14" t="s">
         <v>397</v>
       </c>
-      <c r="D99" s="1"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D99" s="14"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="1"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="3">
         <v>98</v>
       </c>
-      <c r="B100" s="20" t="s">
+      <c r="B100" s="19" t="s">
         <v>398</v>
       </c>
       <c r="C100" s="14" t="s">
         <v>399</v>
       </c>
-      <c r="D100" s="1"/>
-    </row>
-    <row r="101" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D100" s="14"/>
+      <c r="E100" s="14"/>
+      <c r="F100" s="1"/>
+    </row>
+    <row r="101" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A101" s="3">
         <v>99</v>
       </c>
-      <c r="B101" s="20" t="s">
+      <c r="B101" s="19" t="s">
         <v>400</v>
       </c>
       <c r="C101" s="14" t="s">
         <v>401</v>
       </c>
-      <c r="D101" s="1"/>
-    </row>
-    <row r="102" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="D101" s="14"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="1"/>
+    </row>
+    <row r="102" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A102" s="3">
         <v>100</v>
       </c>
-      <c r="B102" s="20" t="s">
+      <c r="B102" s="19" t="s">
         <v>402</v>
       </c>
       <c r="C102" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="D102" s="1"/>
+      <c r="D102" s="14"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C4" r:id="rId1" xr:uid="{45CEC0AE-EA25-4580-80DE-4471360F4FA0}"/>
@@ -5063,23 +5491,25 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{058AFFE3-A0F3-4E80-8D04-89410BA0194C}">
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.33203125" customWidth="1"/>
-    <col min="2" max="2" width="50.6640625" style="21" customWidth="1"/>
-    <col min="3" max="3" width="35.77734375" style="23" customWidth="1"/>
+    <col min="2" max="2" width="50.6640625" style="20" customWidth="1"/>
+    <col min="3" max="5" width="35.77734375" style="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="19.2" x14ac:dyDescent="0.3">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:6" ht="19.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-    </row>
-    <row r="2" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+    </row>
+    <row r="2" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -5090,646 +5520,758 @@
         <v>3</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="39" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" ht="39" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>405</v>
       </c>
-      <c r="D3" s="6"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D3" s="21"/>
+      <c r="E3" s="21"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>2</v>
       </c>
       <c r="B4" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>407</v>
       </c>
-      <c r="D4" s="6"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>3</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>409</v>
       </c>
-      <c r="D5" s="6"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="6"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>4</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>410</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>411</v>
       </c>
-      <c r="D6" s="6"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>412</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="21" t="s">
         <v>413</v>
       </c>
-      <c r="D7" s="6"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D7" s="21"/>
+      <c r="E7" s="21"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>414</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="21" t="s">
         <v>415</v>
       </c>
-      <c r="D8" s="6"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D8" s="21"/>
+      <c r="E8" s="21"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>416</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="21" t="s">
         <v>417</v>
       </c>
-      <c r="D9" s="6"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
         <v>418</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="21" t="s">
         <v>419</v>
       </c>
-      <c r="D10" s="6"/>
-    </row>
-    <row r="11" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D10" s="21"/>
+      <c r="E10" s="21"/>
+      <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
         <v>420</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="21" t="s">
         <v>421</v>
       </c>
-      <c r="D11" s="6"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="6"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>10</v>
       </c>
       <c r="B12" s="7" t="s">
         <v>422</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="21" t="s">
         <v>423</v>
       </c>
-      <c r="D12" s="6"/>
-    </row>
-    <row r="13" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>11</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>424</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="21" t="s">
         <v>425</v>
       </c>
-      <c r="D13" s="6"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>12</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>426</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="21" t="s">
         <v>427</v>
       </c>
-      <c r="D14" s="6"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D14" s="21"/>
+      <c r="E14" s="21"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>13</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>428</v>
       </c>
-      <c r="C15" s="24" t="s">
+      <c r="C15" s="23" t="s">
         <v>429</v>
       </c>
-      <c r="D15" s="6"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D15" s="23"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>14</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>430</v>
       </c>
-      <c r="C16" s="24" t="s">
+      <c r="C16" s="23" t="s">
         <v>431</v>
       </c>
-      <c r="D16" s="6"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D16" s="23"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>432</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="23" t="s">
         <v>433</v>
       </c>
-      <c r="D17" s="6"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D17" s="23"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>434</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="23" t="s">
         <v>435</v>
       </c>
-      <c r="D18" s="6"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D18" s="23"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>436</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="23" t="s">
         <v>437</v>
       </c>
-      <c r="D19" s="6"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D19" s="23"/>
+      <c r="E19" s="23"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>18</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>438</v>
       </c>
-      <c r="C20" s="24" t="s">
+      <c r="C20" s="23" t="s">
         <v>439</v>
       </c>
-      <c r="D20" s="6"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>19</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>440</v>
       </c>
-      <c r="C21" s="24" t="s">
+      <c r="C21" s="23" t="s">
         <v>441</v>
       </c>
-      <c r="D21" s="6"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D21" s="23"/>
+      <c r="E21" s="23"/>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>20</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>442</v>
       </c>
-      <c r="C22" s="24" t="s">
+      <c r="C22" s="23" t="s">
         <v>443</v>
       </c>
-      <c r="D22" s="6"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D22" s="23"/>
+      <c r="E22" s="23"/>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>21</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>444</v>
       </c>
-      <c r="C23" s="24" t="s">
+      <c r="C23" s="23" t="s">
         <v>445</v>
       </c>
-      <c r="D23" s="6"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D23" s="23"/>
+      <c r="E23" s="23"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>22</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>446</v>
       </c>
-      <c r="C24" s="24" t="s">
+      <c r="C24" s="23" t="s">
         <v>447</v>
       </c>
-      <c r="D24" s="6"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D24" s="23"/>
+      <c r="E24" s="23"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>448</v>
       </c>
-      <c r="C25" s="24" t="s">
+      <c r="C25" s="23" t="s">
         <v>449</v>
       </c>
-      <c r="D25" s="6"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D25" s="23"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>24</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>450</v>
       </c>
-      <c r="C26" s="24" t="s">
+      <c r="C26" s="23" t="s">
         <v>451</v>
       </c>
-      <c r="D26" s="6"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D26" s="23"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="6"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>25</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>452</v>
       </c>
-      <c r="C27" s="24" t="s">
+      <c r="C27" s="23" t="s">
         <v>453</v>
       </c>
-      <c r="D27" s="6"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D27" s="23"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="3">
         <v>26</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>454</v>
       </c>
-      <c r="C28" s="24" t="s">
+      <c r="C28" s="23" t="s">
         <v>455</v>
       </c>
-      <c r="D28" s="6"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D28" s="23"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="3">
         <v>27</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>456</v>
       </c>
-      <c r="C29" s="24" t="s">
+      <c r="C29" s="23" t="s">
         <v>457</v>
       </c>
-      <c r="D29" s="6"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D29" s="23"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="3">
         <v>28</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>458</v>
       </c>
-      <c r="C30" s="24" t="s">
+      <c r="C30" s="23" t="s">
         <v>459</v>
       </c>
-      <c r="D30" s="6"/>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D30" s="23"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="3">
         <v>29</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>460</v>
       </c>
-      <c r="C31" s="24" t="s">
+      <c r="C31" s="23" t="s">
         <v>461</v>
       </c>
-      <c r="D31" s="6"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D31" s="23"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="3">
         <v>30</v>
       </c>
       <c r="B32" s="6" t="s">
         <v>462</v>
       </c>
-      <c r="C32" s="24" t="s">
+      <c r="C32" s="23" t="s">
         <v>463</v>
       </c>
-      <c r="D32" s="6"/>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D32" s="23"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="3">
         <v>31</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>464</v>
       </c>
-      <c r="C33" s="24" t="s">
+      <c r="C33" s="23" t="s">
         <v>465</v>
       </c>
-      <c r="D33" s="6"/>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D33" s="23"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="3">
         <v>32</v>
       </c>
       <c r="B34" s="7" t="s">
         <v>467</v>
       </c>
-      <c r="C34" s="24" t="s">
+      <c r="C34" s="23" t="s">
         <v>466</v>
       </c>
-      <c r="D34" s="6"/>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D34" s="23"/>
+      <c r="E34" s="23"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="3">
         <v>33</v>
       </c>
       <c r="B35" s="7" t="s">
         <v>468</v>
       </c>
-      <c r="C35" s="24" t="s">
+      <c r="C35" s="23" t="s">
         <v>469</v>
       </c>
-      <c r="D35" s="6"/>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D35" s="23"/>
+      <c r="E35" s="23"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="3">
         <v>34</v>
       </c>
       <c r="B36" s="7" t="s">
         <v>470</v>
       </c>
-      <c r="C36" s="24" t="s">
+      <c r="C36" s="23" t="s">
         <v>471</v>
       </c>
-      <c r="D36" s="6"/>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D36" s="23"/>
+      <c r="E36" s="23"/>
+      <c r="F36" s="6"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="3">
         <v>35</v>
       </c>
       <c r="B37" s="7" t="s">
         <v>472</v>
       </c>
-      <c r="C37" s="24" t="s">
+      <c r="C37" s="23" t="s">
         <v>473</v>
       </c>
-      <c r="D37" s="6"/>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
+      <c r="F37" s="6"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="3">
         <v>36</v>
       </c>
       <c r="B38" s="7" t="s">
         <v>474</v>
       </c>
-      <c r="C38" s="24" t="s">
+      <c r="C38" s="23" t="s">
         <v>475</v>
       </c>
-      <c r="D38" s="6"/>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D38" s="23"/>
+      <c r="E38" s="23"/>
+      <c r="F38" s="6"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="3">
         <v>37</v>
       </c>
       <c r="B39" s="7" t="s">
         <v>476</v>
       </c>
-      <c r="C39" s="24" t="s">
+      <c r="C39" s="23" t="s">
         <v>477</v>
       </c>
-      <c r="D39" s="6"/>
-    </row>
-    <row r="40" spans="1:4" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D39" s="23"/>
+      <c r="E39" s="23"/>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" spans="1:6" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3">
         <v>38</v>
       </c>
       <c r="B40" s="7" t="s">
         <v>478</v>
       </c>
-      <c r="C40" s="24" t="s">
+      <c r="C40" s="23" t="s">
         <v>479</v>
       </c>
-      <c r="D40" s="6"/>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D40" s="23"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="6"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="3">
         <v>39</v>
       </c>
       <c r="B41" s="7" t="s">
         <v>480</v>
       </c>
-      <c r="C41" s="24" t="s">
+      <c r="C41" s="23" t="s">
         <v>481</v>
       </c>
-      <c r="D41" s="6"/>
-    </row>
-    <row r="42" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D41" s="23"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="6"/>
+    </row>
+    <row r="42" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A42" s="3">
         <v>40</v>
       </c>
       <c r="B42" s="7" t="s">
         <v>482</v>
       </c>
-      <c r="C42" s="24" t="s">
+      <c r="C42" s="23" t="s">
         <v>483</v>
       </c>
-      <c r="D42" s="6"/>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D42" s="23"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="6"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="3">
         <v>41</v>
       </c>
       <c r="B43" s="7" t="s">
         <v>484</v>
       </c>
-      <c r="C43" s="24" t="s">
+      <c r="C43" s="23" t="s">
         <v>485</v>
       </c>
-      <c r="D43" s="6"/>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D43" s="23"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="6"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="3">
         <v>42</v>
       </c>
       <c r="B44" s="7" t="s">
         <v>486</v>
       </c>
-      <c r="C44" s="24" t="s">
+      <c r="C44" s="23" t="s">
         <v>487</v>
       </c>
-      <c r="D44" s="6"/>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D44" s="23"/>
+      <c r="E44" s="23"/>
+      <c r="F44" s="6"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="3">
         <v>43</v>
       </c>
       <c r="B45" s="7" t="s">
         <v>488</v>
       </c>
-      <c r="C45" s="24" t="s">
+      <c r="C45" s="23" t="s">
         <v>489</v>
       </c>
-      <c r="D45" s="6"/>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D45" s="23"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="6"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="3">
         <v>44</v>
       </c>
       <c r="B46" s="7" t="s">
         <v>490</v>
       </c>
-      <c r="C46" s="24" t="s">
+      <c r="C46" s="23" t="s">
         <v>491</v>
       </c>
-      <c r="D46" s="6"/>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D46" s="23"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="6"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="3">
         <v>45</v>
       </c>
       <c r="B47" s="7" t="s">
         <v>492</v>
       </c>
-      <c r="C47" s="24" t="s">
+      <c r="C47" s="23" t="s">
         <v>493</v>
       </c>
-      <c r="D47" s="6"/>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D47" s="23"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="6"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="3">
         <v>46</v>
       </c>
       <c r="B48" s="7" t="s">
         <v>494</v>
       </c>
-      <c r="C48" s="24" t="s">
+      <c r="C48" s="23" t="s">
         <v>495</v>
       </c>
-      <c r="D48" s="6"/>
-    </row>
-    <row r="49" spans="1:4" ht="26.4" x14ac:dyDescent="0.3">
+      <c r="D48" s="23"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="6"/>
+    </row>
+    <row r="49" spans="1:6" ht="26.4" x14ac:dyDescent="0.3">
       <c r="A49" s="3">
         <v>47</v>
       </c>
       <c r="B49" s="7" t="s">
         <v>497</v>
       </c>
-      <c r="C49" s="24" t="s">
+      <c r="C49" s="23" t="s">
         <v>496</v>
       </c>
-      <c r="D49" s="6"/>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D49" s="23"/>
+      <c r="E49" s="23"/>
+      <c r="F49" s="6"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="3">
         <v>48</v>
       </c>
       <c r="B50" s="7" t="s">
         <v>498</v>
       </c>
-      <c r="C50" s="24" t="s">
+      <c r="C50" s="23" t="s">
         <v>499</v>
       </c>
-      <c r="D50" s="6"/>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D50" s="23"/>
+      <c r="E50" s="23"/>
+      <c r="F50" s="6"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="3">
         <v>49</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>501</v>
       </c>
-      <c r="C51" s="24" t="s">
+      <c r="C51" s="23" t="s">
         <v>500</v>
       </c>
-      <c r="D51" s="6"/>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D51" s="23"/>
+      <c r="E51" s="23"/>
+      <c r="F51" s="6"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="3">
         <v>50</v>
       </c>
       <c r="B52" s="7" t="s">
         <v>502</v>
       </c>
-      <c r="C52" s="24" t="s">
+      <c r="C52" s="23" t="s">
         <v>503</v>
       </c>
-      <c r="D52" s="6"/>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D52" s="23"/>
+      <c r="E52" s="23"/>
+      <c r="F52" s="6"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="3">
         <v>51</v>
       </c>
       <c r="B53" s="7" t="s">
         <v>504</v>
       </c>
-      <c r="C53" s="24" t="s">
+      <c r="C53" s="23" t="s">
         <v>505</v>
       </c>
-      <c r="D53" s="6"/>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D53" s="23"/>
+      <c r="E53" s="23"/>
+      <c r="F53" s="6"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="3">
         <v>52</v>
       </c>
       <c r="B54" s="7" t="s">
         <v>506</v>
       </c>
-      <c r="C54" s="24" t="s">
+      <c r="C54" s="23" t="s">
         <v>507</v>
       </c>
-      <c r="D54" s="6"/>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D54" s="23"/>
+      <c r="E54" s="23"/>
+      <c r="F54" s="6"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="3">
         <v>53</v>
       </c>
       <c r="B55" s="7" t="s">
         <v>508</v>
       </c>
-      <c r="C55" s="24" t="s">
+      <c r="C55" s="23" t="s">
         <v>509</v>
       </c>
-      <c r="D55" s="6"/>
-    </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D55" s="23"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="6"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="3">
         <v>54</v>
       </c>
@@ -5739,9 +6281,11 @@
       <c r="C56" s="9" t="s">
         <v>511</v>
       </c>
-      <c r="D56" s="6"/>
-    </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D56" s="9"/>
+      <c r="E56" s="9"/>
+      <c r="F56" s="6"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="3">
         <v>55</v>
       </c>
@@ -5751,9 +6295,11 @@
       <c r="C57" t="s">
         <v>512</v>
       </c>
-      <c r="D57" s="7"/>
-    </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D57"/>
+      <c r="E57"/>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="3">
         <v>56</v>
       </c>
@@ -5763,9 +6309,11 @@
       <c r="C58" t="s">
         <v>513</v>
       </c>
-      <c r="D58" s="7"/>
-    </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D58"/>
+      <c r="E58"/>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="3">
         <v>57</v>
       </c>
@@ -5775,9 +6323,11 @@
       <c r="C59" t="s">
         <v>514</v>
       </c>
-      <c r="D59" s="7"/>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D59"/>
+      <c r="E59"/>
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="3">
         <v>58</v>
       </c>
@@ -5787,9 +6337,11 @@
       <c r="C60" t="s">
         <v>516</v>
       </c>
-      <c r="D60" s="7"/>
-    </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D60"/>
+      <c r="E60"/>
+      <c r="F60" s="7"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="3">
         <v>59</v>
       </c>
@@ -5799,9 +6351,11 @@
       <c r="C61" t="s">
         <v>517</v>
       </c>
-      <c r="D61" s="7"/>
-    </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D61"/>
+      <c r="E61"/>
+      <c r="F61" s="7"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="3">
         <v>60</v>
       </c>
@@ -5811,9 +6365,11 @@
       <c r="C62" t="s">
         <v>518</v>
       </c>
-      <c r="D62" s="7"/>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D62"/>
+      <c r="E62"/>
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="3">
         <v>61</v>
       </c>
@@ -5823,9 +6379,11 @@
       <c r="C63" t="s">
         <v>519</v>
       </c>
-      <c r="D63" s="7"/>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D63"/>
+      <c r="E63"/>
+      <c r="F63" s="7"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="3">
         <v>62</v>
       </c>
@@ -5835,9 +6393,11 @@
       <c r="C64" t="s">
         <v>520</v>
       </c>
-      <c r="D64" s="7"/>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D64"/>
+      <c r="E64"/>
+      <c r="F64" s="7"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="3">
         <v>63</v>
       </c>
@@ -5847,9 +6407,11 @@
       <c r="C65" t="s">
         <v>521</v>
       </c>
-      <c r="D65" s="7"/>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D65"/>
+      <c r="E65"/>
+      <c r="F65" s="7"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="3">
         <v>64</v>
       </c>
@@ -5859,9 +6421,11 @@
       <c r="C66" t="s">
         <v>522</v>
       </c>
-      <c r="D66" s="7"/>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D66"/>
+      <c r="E66"/>
+      <c r="F66" s="7"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="3">
         <v>65</v>
       </c>
@@ -5871,9 +6435,11 @@
       <c r="C67" t="s">
         <v>524</v>
       </c>
-      <c r="D67" s="7"/>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D67"/>
+      <c r="E67"/>
+      <c r="F67" s="7"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="3">
         <v>66</v>
       </c>
@@ -5883,9 +6449,11 @@
       <c r="C68" t="s">
         <v>525</v>
       </c>
-      <c r="D68" s="7"/>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D68"/>
+      <c r="E68"/>
+      <c r="F68" s="7"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="3">
         <v>67</v>
       </c>
@@ -5895,9 +6463,11 @@
       <c r="C69" t="s">
         <v>526</v>
       </c>
-      <c r="D69" s="7"/>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D69"/>
+      <c r="E69"/>
+      <c r="F69" s="7"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="3">
         <v>68</v>
       </c>
@@ -5907,9 +6477,11 @@
       <c r="C70" t="s">
         <v>527</v>
       </c>
-      <c r="D70" s="7"/>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D70"/>
+      <c r="E70"/>
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="3">
         <v>69</v>
       </c>
@@ -5919,9 +6491,11 @@
       <c r="C71" t="s">
         <v>528</v>
       </c>
-      <c r="D71" s="7"/>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D71"/>
+      <c r="E71"/>
+      <c r="F71" s="7"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="3">
         <v>70</v>
       </c>
@@ -5931,9 +6505,11 @@
       <c r="C72" t="s">
         <v>529</v>
       </c>
-      <c r="D72" s="7"/>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D72"/>
+      <c r="E72"/>
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="3">
         <v>71</v>
       </c>
@@ -5943,9 +6519,11 @@
       <c r="C73" t="s">
         <v>530</v>
       </c>
-      <c r="D73" s="1"/>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D73"/>
+      <c r="E73"/>
+      <c r="F73" s="1"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="3">
         <v>72</v>
       </c>
@@ -5955,9 +6533,11 @@
       <c r="C74" t="s">
         <v>531</v>
       </c>
-      <c r="D74" s="1"/>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D74"/>
+      <c r="E74"/>
+      <c r="F74" s="1"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="3">
         <v>73</v>
       </c>
@@ -5967,9 +6547,11 @@
       <c r="C75" t="s">
         <v>532</v>
       </c>
-      <c r="D75" s="1"/>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D75"/>
+      <c r="E75"/>
+      <c r="F75" s="1"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="3">
         <v>74</v>
       </c>
@@ -5979,9 +6561,11 @@
       <c r="C76" t="s">
         <v>533</v>
       </c>
-      <c r="D76" s="1"/>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D76"/>
+      <c r="E76"/>
+      <c r="F76" s="1"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="3">
         <v>75</v>
       </c>
@@ -5991,9 +6575,11 @@
       <c r="C77" t="s">
         <v>534</v>
       </c>
-      <c r="D77" s="1"/>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D77"/>
+      <c r="E77"/>
+      <c r="F77" s="1"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="3">
         <v>76</v>
       </c>
@@ -6003,9 +6589,11 @@
       <c r="C78" t="s">
         <v>535</v>
       </c>
-      <c r="D78" s="1"/>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D78"/>
+      <c r="E78"/>
+      <c r="F78" s="1"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="3">
         <v>77</v>
       </c>
@@ -6015,9 +6603,11 @@
       <c r="C79" t="s">
         <v>536</v>
       </c>
-      <c r="D79" s="1"/>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D79"/>
+      <c r="E79"/>
+      <c r="F79" s="1"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="3">
         <v>78</v>
       </c>
@@ -6027,9 +6617,11 @@
       <c r="C80" t="s">
         <v>537</v>
       </c>
-      <c r="D80" s="1"/>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D80"/>
+      <c r="E80"/>
+      <c r="F80" s="1"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="3">
         <v>79</v>
       </c>
@@ -6039,9 +6631,11 @@
       <c r="C81" t="s">
         <v>538</v>
       </c>
-      <c r="D81" s="1"/>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D81"/>
+      <c r="E81"/>
+      <c r="F81" s="1"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="3">
         <v>80</v>
       </c>
@@ -6051,9 +6645,11 @@
       <c r="C82" t="s">
         <v>539</v>
       </c>
-      <c r="D82" s="1"/>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D82"/>
+      <c r="E82"/>
+      <c r="F82" s="1"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="3">
         <v>81</v>
       </c>
@@ -6063,9 +6659,11 @@
       <c r="C83" t="s">
         <v>540</v>
       </c>
-      <c r="D83" s="1"/>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D83"/>
+      <c r="E83"/>
+      <c r="F83" s="1"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="3">
         <v>82</v>
       </c>
@@ -6075,9 +6673,11 @@
       <c r="C84" t="s">
         <v>541</v>
       </c>
-      <c r="D84" s="1"/>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D84"/>
+      <c r="E84"/>
+      <c r="F84" s="1"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="3">
         <v>83</v>
       </c>
@@ -6087,9 +6687,11 @@
       <c r="C85" t="s">
         <v>543</v>
       </c>
-      <c r="D85" s="1"/>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D85"/>
+      <c r="E85"/>
+      <c r="F85" s="1"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="3">
         <v>84</v>
       </c>
@@ -6099,9 +6701,11 @@
       <c r="C86" t="s">
         <v>544</v>
       </c>
-      <c r="D86" s="1"/>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D86"/>
+      <c r="E86"/>
+      <c r="F86" s="1"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="3">
         <v>85</v>
       </c>
@@ -6111,9 +6715,11 @@
       <c r="C87" t="s">
         <v>545</v>
       </c>
-      <c r="D87" s="1"/>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D87"/>
+      <c r="E87"/>
+      <c r="F87" s="1"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="3">
         <v>86</v>
       </c>
@@ -6123,9 +6729,11 @@
       <c r="C88" t="s">
         <v>546</v>
       </c>
-      <c r="D88" s="1"/>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D88"/>
+      <c r="E88"/>
+      <c r="F88" s="1"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="3">
         <v>87</v>
       </c>
@@ -6135,9 +6743,11 @@
       <c r="C89" t="s">
         <v>547</v>
       </c>
-      <c r="D89" s="1"/>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D89"/>
+      <c r="E89"/>
+      <c r="F89" s="1"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="3">
         <v>88</v>
       </c>
@@ -6147,9 +6757,11 @@
       <c r="C90" t="s">
         <v>548</v>
       </c>
-      <c r="D90" s="1"/>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D90"/>
+      <c r="E90"/>
+      <c r="F90" s="1"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="3">
         <v>89</v>
       </c>
@@ -6159,9 +6771,11 @@
       <c r="C91" t="s">
         <v>549</v>
       </c>
-      <c r="D91" s="1"/>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D91"/>
+      <c r="E91"/>
+      <c r="F91" s="1"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="3">
         <v>90</v>
       </c>
@@ -6171,9 +6785,11 @@
       <c r="C92" t="s">
         <v>550</v>
       </c>
-      <c r="D92" s="1"/>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D92"/>
+      <c r="E92"/>
+      <c r="F92" s="1"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="3">
         <v>91</v>
       </c>
@@ -6183,9 +6799,11 @@
       <c r="C93" t="s">
         <v>551</v>
       </c>
-      <c r="D93" s="1"/>
-    </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D93"/>
+      <c r="E93"/>
+      <c r="F93" s="1"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="3">
         <v>92</v>
       </c>
@@ -6195,9 +6813,11 @@
       <c r="C94" t="s">
         <v>552</v>
       </c>
-      <c r="D94" s="1"/>
-    </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D94"/>
+      <c r="E94"/>
+      <c r="F94" s="1"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="3">
         <v>93</v>
       </c>
@@ -6207,9 +6827,11 @@
       <c r="C95" t="s">
         <v>553</v>
       </c>
-      <c r="D95" s="1"/>
-    </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D95"/>
+      <c r="E95"/>
+      <c r="F95" s="1"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="3">
         <v>94</v>
       </c>
@@ -6219,9 +6841,11 @@
       <c r="C96" t="s">
         <v>554</v>
       </c>
-      <c r="D96" s="1"/>
-    </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D96"/>
+      <c r="E96"/>
+      <c r="F96" s="1"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="3">
         <v>95</v>
       </c>
@@ -6231,9 +6855,11 @@
       <c r="C97" t="s">
         <v>555</v>
       </c>
-      <c r="D97" s="1"/>
-    </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D97"/>
+      <c r="E97"/>
+      <c r="F97" s="1"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="3">
         <v>96</v>
       </c>
@@ -6243,9 +6869,11 @@
       <c r="C98" t="s">
         <v>556</v>
       </c>
-      <c r="D98" s="1"/>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D98"/>
+      <c r="E98"/>
+      <c r="F98" s="1"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="3">
         <v>97</v>
       </c>
@@ -6255,9 +6883,11 @@
       <c r="C99" t="s">
         <v>557</v>
       </c>
-      <c r="D99" s="1"/>
-    </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D99"/>
+      <c r="E99"/>
+      <c r="F99" s="1"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="3">
         <v>98</v>
       </c>
@@ -6267,9 +6897,11 @@
       <c r="C100" t="s">
         <v>559</v>
       </c>
-      <c r="D100" s="1"/>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D100"/>
+      <c r="E100"/>
+      <c r="F100" s="1"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="3">
         <v>99</v>
       </c>
@@ -6279,9 +6911,11 @@
       <c r="C101" t="s">
         <v>560</v>
       </c>
-      <c r="D101" s="1"/>
-    </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D101"/>
+      <c r="E101"/>
+      <c r="F101" s="1"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="3">
         <v>100</v>
       </c>
@@ -6291,15 +6925,19 @@
       <c r="C102" t="s">
         <v>561</v>
       </c>
-      <c r="D102" s="1"/>
-    </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D102"/>
+      <c r="E102"/>
+      <c r="F102" s="1"/>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B103"/>
       <c r="C103"/>
+      <c r="D103"/>
+      <c r="E103"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="C3" r:id="rId1" xr:uid="{C6A8AF16-E57C-4730-9DB6-0A3A5E36643C}"/>

</xml_diff>

<commit_message>
Doc duoc moi sheet Excel, bao ro sheet nao bi bo qua
- findHeader nhan cot ten linh hoat (Ten san pham / Ten shop / Ten SP)
  thay vi chi dung "Ten san pham", nen sheet "Shop quan ao" khong con bi bo
- parseCatalogXlsx tra them skipped: ten sheet + ly do bi bo qua
- Popup hien dong "Bo qua N sheet: ... - ly do" va so version dang chay,
  tooltip version cho biet Chrome dang load thu muc extension nao
- Bump version 2.0.0 -> 2.1.0

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PygyS4qjo2M4C3NBeKaChU
</commit_message>
<xml_diff>
--- a/data/seeding.xlsx
+++ b/data/seeding.xlsx
@@ -5,17 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\freelancer\baotran\affliate-comment\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Seeding-media\comment-thread\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E919DBF-FD03-4FDB-8676-A43EC8B2B593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB88F9B0-0C06-424E-B20A-64CF8DB64F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FB351C2D-D222-4FD7-8A1F-0AFAF061EB0D}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="14016" windowHeight="13056" firstSheet="1" activeTab="3" xr2:uid="{FB351C2D-D222-4FD7-8A1F-0AFAF061EB0D}"/>
   </bookViews>
   <sheets>
     <sheet name="Chăm sóc da mặt - body " sheetId="1" r:id="rId1"/>
     <sheet name="Trang điểm" sheetId="3" r:id="rId2"/>
     <sheet name="Ăn uống" sheetId="4" r:id="rId3"/>
+    <sheet name="Thời trang" sheetId="6" r:id="rId4"/>
+    <sheet name="Shop quần áo" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="608">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="876" uniqueCount="842">
   <si>
     <t>Link rút gọn - CHĂM SÓC DA</t>
   </si>
@@ -1875,6 +1877,708 @@
   </si>
   <si>
     <t>giá</t>
+  </si>
+  <si>
+    <t>Link rút gọn - Quần áo</t>
+  </si>
+  <si>
+    <t>ICON DENIM</t>
+  </si>
+  <si>
+    <t>Tên shop</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3B7SgriDF1</t>
+  </si>
+  <si>
+    <t>chuyên quần áo nam</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1qc56TJtpy</t>
+  </si>
+  <si>
+    <t>NEVO Sport</t>
+  </si>
+  <si>
+    <t>thời trang thể thao</t>
+  </si>
+  <si>
+    <t>ViettienStore</t>
+  </si>
+  <si>
+    <t>đồ văn phòng nam</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/80CiRu8A43</t>
+  </si>
+  <si>
+    <t>ONOFF by RE:ON</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3g3jHzmKeJ</t>
+  </si>
+  <si>
+    <t>Shop đồ lót nam nữ</t>
+  </si>
+  <si>
+    <t>VISECRET_BRA</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3VkJ5jupT3</t>
+  </si>
+  <si>
+    <t>Shop đồ lót nữ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7ptIFpsYvZ</t>
+  </si>
+  <si>
+    <t>Rayban</t>
+  </si>
+  <si>
+    <t>kính mát</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/40gZgqAgf5</t>
+  </si>
+  <si>
+    <t>MEIXUEMEILIN</t>
+  </si>
+  <si>
+    <t>thời trang nữ</t>
+  </si>
+  <si>
+    <t>Thời trang thể thao Dunlop</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1VzEiLutfr</t>
+  </si>
+  <si>
+    <t>Thời trang thể thao</t>
+  </si>
+  <si>
+    <t>FILA Việt Nam</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3LQstqgDY3</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8fSPFhlmua</t>
+  </si>
+  <si>
+    <t>Kosu Shoesinjapan</t>
+  </si>
+  <si>
+    <t>Giày dép nữ</t>
+  </si>
+  <si>
+    <t>Pier N05 &amp; SantonY</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2VrluToM97</t>
+  </si>
+  <si>
+    <t>Đồ lót nữ</t>
+  </si>
+  <si>
+    <t>GUZADO MENSWEAR</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8V8z3YiWKG</t>
+  </si>
+  <si>
+    <t>Thời trang nam</t>
+  </si>
+  <si>
+    <t>MUTU 慕兔</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/112y7pHu5m</t>
+  </si>
+  <si>
+    <t>Thời trang nữ</t>
+  </si>
+  <si>
+    <t>JBAGY _ Official Store</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2qUcJHQR10</t>
+  </si>
+  <si>
+    <t>Đồ lót nam nữ ROCK annie</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/gQ7jNSC8p</t>
+  </si>
+  <si>
+    <t>Đồ lót nam nữ</t>
+  </si>
+  <si>
+    <t>ONOFF Official Store</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2qUcJPBzvk</t>
+  </si>
+  <si>
+    <t>Cillie Official</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1LfoWipI2W</t>
+  </si>
+  <si>
+    <t>Bevis Store</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/905Feqjq0b</t>
+  </si>
+  <si>
+    <t>Phụ kiện thời trang</t>
+  </si>
+  <si>
+    <t>Thời Trang Nam MIKOFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thời Trang Nam </t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/30o2Vrs8As</t>
+  </si>
+  <si>
+    <t>Winfit</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7ptIGnyuwM</t>
+  </si>
+  <si>
+    <t>Urban Revivo</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/W6hXTwKPB</t>
+  </si>
+  <si>
+    <t>Thời Trang Nam Nữ</t>
+  </si>
+  <si>
+    <t>Owen Official Store</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1gIevg4HpH</t>
+  </si>
+  <si>
+    <t>Thời Trang Nam</t>
+  </si>
+  <si>
+    <t>Dwin Official Store</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AAHD3LNdpV</t>
+  </si>
+  <si>
+    <t>Đồ bộ mặc nhà cao cấp Sunfly</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3g3jJS333o</t>
+  </si>
+  <si>
+    <t>Đồ bộ mặc nhà cao cấp</t>
+  </si>
+  <si>
+    <t>IVY moda</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2qUcJxaYS4</t>
+  </si>
+  <si>
+    <t>CAVERA ATELIER Vietnam</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/6q0l5S0ELM</t>
+  </si>
+  <si>
+    <t>Coolmate - Official Store</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3VkJ7NgVRq</t>
+  </si>
+  <si>
+    <t>Guzado Official</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3VkJ7QWDgd</t>
+  </si>
+  <si>
+    <t>Đầm bẹt vai</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8KpYt342Nt</t>
+  </si>
+  <si>
+    <t>Đầm soắn ngực</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8AW8gk4fis</t>
+  </si>
+  <si>
+    <t>Đầm nhung khoét vai</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/80CiUR5J3r</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9AOfsa0rh6</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/905FgH1V25</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8plpTy28N4</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8fSPHf2li3</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9peMfnyKLI</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9fKwTUyxgH</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9V1WHBzb1G</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9Ki64t0EMF</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AUu3T1vmzU</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AKadGiwQKT</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AAHD4Px3fS</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9zxms6xh0R</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/5q8DuSDYSe</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/5foni9EBnd</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/5VVNVqEp8c</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/5LBxJXFSTb</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/6VNuhgB16q</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/6L4UVNBeRp</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/6Al4J4CHmo</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/60Re6lCv7n</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7AdbUu8Tl2</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/70KBIb9761</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/6q0l6I9kR0</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/6fhKtzANlz</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7ptII85wPE</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7fZs5p6ZkD</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7VGRtW7D5C</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/7Kx1hD7qQB</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3B7SjYNhsO</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/30o2XFOLDN</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2qUcKwOyYM</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2gBC8dPbtL</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3qN9WmLAWa</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3g3jKTLnrZ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3VkJ8AMRCY</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/3LQsvrN4XX</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Hai Dây Lụa Phi Bóng Hồng Baby Phối Ren Nơ Tiểu Thư Đi Biển Mùa Hè</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/4VcqK0IdAm</t>
+  </si>
+  <si>
+    <t>| LYN WEAR| ( HOẢ TỐC) Đầm Ôm Body Sọc Len Sát Nách Nữ Dáng Dài Tối Giản Thanh Lịch Đi Làm Đi Tiệc</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/4LJQ7hJGVl</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) ĐẦM BODY HỒNG PASTEL TAY DÀI CỔ VUÔNG HÀN QUỐC</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/4AzzvOJtqk</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm cổ xoắn form xòe MPB.Váy body nữ trễ vai basic đi chơi, đi tiệc sang chảnh mùa hè.</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/40gZj5KXBj</t>
+  </si>
+  <si>
+    <t>[ SUMMER TOP ] (HOẢ TỐC) Áo Babydoll 2 Dây Nữ Dáng Xòe Xinh – Thiết Kế Khoét Giữa Dễ Thương Đi Chơi Đi Biển</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/5AsX7EG5oy</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Hai Dây Nữ Bí Tơ Phối Ren Cách Điệu Cúp Ngực Dáng Xòe Baby Doll Màu Trắng Freesize</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/50Z6uvGj9x</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (DEAL MỞ BÁN) Đầm Nữ Cổ Viền Form Xòe Dáng Ôm Nhẹ Tôn Dáng Thanh Lịch</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/4qFgicHMUw</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm Xòe Hai Dây Bản To Phối Nơ Nữ Form Baby Doll Tôn Dáng Đi Biển Đi Chơi</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/4fwGWJHzpv</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm Xòe Đen Cổ Vuông Hai Dây Bản To Ôm Eo Tôn Dáng Váy Ngắn Nữ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/W6hYeXrI8</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm Xòe Len Sọc Loại 1 Sát Nách Ôm Body | Khóa Kéo Sau, Mỏng Nhẹ, Tôn Dáng</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/LnHMLYUd7</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm Body 2 Dây Nhún Ngực Tôn V1 – Váy Ôm Body Thun Rip Trung Mỏng Nhẹ, Không Nóng</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/BTrA2Z7y6</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm Nữ Cổ Lọ Form Xoè Dáng Ngắn – Tôn Dáng, Mặc Đi Chơi Đi Tiệc</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1AQxjZlJ5</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm ôm body sát nách thun rip Trung mịn mát, đầm Basic màu đen dễ phối.</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1BMOLsVJwK</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Kiểu Nữ Coquette Cổ Vuông Tay Phồng Nơ Eo Dáng Peplum</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/112y9ZVxHJ</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HỎA TỐC) Đầm Body Nhún Ôm Ngực Tôn Dáng – Váy Body Dự Tiệc Sexy Gợi Cảm</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/qjXxGWacI</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (SUMMER TOP) Áo Hai Dây Nữ basic ôm body rip lụa mềm mịn mát – Nhiều Màu</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/gQ7kxXDxH</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Bodysuit Nữ Dây Đeo Tháo Rời Ôm Dáng Tôn Eo Không Đường May, Nâng Form Mượt Mịn</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1qc596SmaW</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Đầm xoắn ngực tôn dáng. Chất rip lụa ôm eo, mịn mát</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1gIewnTPvV</t>
+  </si>
+  <si>
+    <t>| LYN Wear | (HOẢ TỐC) Áo Ren Kiểu sát Nách Cổ V 2 Màu Đen Trắng Thiết Kế Sang Trọng Phong Cách Thời Trang</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1VzEkUU3GU</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Ống Sọc Dây Yếm Form Ôm Nữ – Thiết Kế Thời Trang Cá Tính</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/1LfoYBUgbT</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Chân Váy Lụa Chữ A Ngắn Xòe Y2K Cạp Thấp Mềm Mịn Nữ Hàn Quốc</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2VrlwKQFEi</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HỎA TỐC) Đầm Ren Nữ 2 Dây Cổ Yếm Dáng Ôm Phối Ren Nữ Tính, Chất đẹp, dày dặn.</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2LYLk1QsZh</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (HOẢ TỐC) Áo Thun Nữ Cổ Tim Chữ V Nhún Ngực Chiết Eo Form Ôm Slim Fit Thun Rib Co Giãn</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/2BEvXiRVug</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | ( HOẢ TỐC)Áo Thun Nữ Trễ Vai Thắt Nơ Tay Ôm Body Cotton Mịn Hàn Quốc</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/20vVLPS9Ff</t>
+  </si>
+  <si>
+    <t>| LYN WEAR| Áo 2 Dây Viền Ren KÈM MÚT, Thun Rip Trung Co Giãn Ôm Form Mềm Mịn Mát</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8KpYt342Ou</t>
+  </si>
+  <si>
+    <t>| LYN WEAR| (HOẢ TỐC-XẢ KHO) Áo ống/ Quây xoắn ngực  Không Mút Chất Cotton Mịn</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8V8z5M3P3x</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Thun Nữ Cổ Tim Nhún Ngực Kẻ Sọc – Dáng Ôm Body, Co Giãn, Tôn Dáng, Mặc Đi Chơi</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/80CiUR5J4s</t>
+  </si>
+  <si>
+    <t>| LYN.WEAR | Đầm Lụa Hai Dây Đính Đá Đuôi Cá Dáng Dài Đi Chơi Dạo Phố Sang Chảnh Tết, Noel, du lịch</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8AW8gk4fjv</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo hai dây cổ đổ thun giấy mùa hè, croptop basic dáng sexy</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/905FgH1V36</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Đầm Ba Lỗ Dáng Xòe Nữ D62 Thời Trang Dễ Mặc Dễ Phối Đồ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9AOfsa0ri9</t>
+  </si>
+  <si>
+    <t>| LYN.WEAR | Chân Váy Tơ Linen Xòe Dáng Dài Nữ Cạp Trễ Phong Cách Nàng Thơ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8fSPHf2lj4</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Ống Nữ Tube Basic | Dễ Phối Thời Trang</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/8plpTy28O7</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo Babydoll Nữ Cổ V Phối Ren Xếp Tầng Tay Ngắn Dáng Xòe</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9fKwTUyxhI</t>
+  </si>
+  <si>
+    <t>| LYN.WEAR | (KÈM QUẦN) Đầm Voan Tơ Babydoll Hai Dây Dáng Bí Vàng Phối Nơ Kim Sa</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9peMfnyKML</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | (MẶC ĐƯỢC 2 KIỂU) Áo Lụa Nữ Trễ Vai-Tay Bèo Lưng Thun, Khoá Kéo Bên Hông Ôm Dáng 5 Màu</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9Ki64t0ENG</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Áo khoác sơ mi trắng nữ form rộng tay dài vạt bầu đũi voan xước mỏng nhẹ đi biển</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9V1WHBzb2J</t>
+  </si>
+  <si>
+    <t>| LYN.WEAR | Set Áo Cổ Tàu Khoét Giọt Nước Kèm Chân Váy Midi Nhún Hồng Pastel Xanh Baby</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AKadGiwQLU</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Đầm Ba Lỗ Ôm Body Nữ Basic Vải Thun Cotton Co Giãn Dễ Mặc Dễ Phối Đồ</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AUu3T1vn0X</t>
+  </si>
+  <si>
+    <t>| LYN WEAR | Đầm Cổ Yếm Dáng Xoè Phối Ren Tôn Dáng Nữ Dáng Ôm Thời Trang Hồng Pastel</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/9zxms6xh1S</t>
+  </si>
+  <si>
+    <t>https://s.shopee.vn/AAHD4Px3gV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo Kiểu Ngắn Tay Rút Eo Thắt Nơ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set áo hai dây layer phối chân váy/quần ống rộng </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Set Áo Thun Kèm Yếm Chấm Bi Thắt Nơ Nhún Bèo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo gile dệt kim nữ cổ V phối khăn thời trang </t>
+  </si>
+  <si>
+    <t>Áo Kiểu Nữ Kẻ Caro Đan Dây Ngực</t>
+  </si>
+  <si>
+    <t>ÁO KIỂU CỔ BÈO ĐÍNH NƠ DÁNG PHỒNG</t>
+  </si>
+  <si>
+    <t>Áo Thun Len Tăm Cổ V Cài Cúc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo Thun Nữ Croptop </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo Kiểu Nữ Gân Rút Nhún Đính Nơ Xinh Xắn </t>
+  </si>
+  <si>
+    <t>Áo Kiểu Sát Nách Giả Hai Mảnh Loang Màu</t>
+  </si>
+  <si>
+    <t>Miếng Dán Cố Định Quần Áo Trong Suốt</t>
+  </si>
+  <si>
+    <t>Hộp 60 Miếng Dán Giấy Hình Hoa</t>
+  </si>
+  <si>
+    <t>Áo Đúc Su Mềm Mịn Nhẹ Nhàng</t>
+  </si>
+  <si>
+    <t>Miếng Dán Ngực Silicon Không Lộ Viền Tệp Da</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Miếng Dán Độn Vai Cho Nam Nữ Nâng Vai </t>
+  </si>
+  <si>
+    <t>QUẦN LỬNG KAKI BERMUDA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bộ thời trang nữ Âu Mỹ </t>
+  </si>
+  <si>
+    <t>Áo Phông Lệch Vai Phối Kẻ Sọc Kristy Boutique</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> [KRISTY BOUTIQUE] ÁO KIỂU REN CỔ V THẮT NƠ </t>
+  </si>
+  <si>
+    <t>#Áo Thun Baby Tee Chấm Bi Phối Nơ</t>
+  </si>
+  <si>
+    <t>QUẦN LỬNG HACK DÁNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Áo Phông Nữ Cổ Tim Giả 2 Dây</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Áo Thun Zip Nữ Form Ôm Tôn Dáng</t>
+  </si>
+  <si>
+    <t>ÁO HAI DÂY CHẤM BI VIỀN REN</t>
+  </si>
+  <si>
+    <t>CHÂN VÁY NGẮN CÓ QUẦN TRONG</t>
+  </si>
+  <si>
+    <t>QUẦN SHORTS JEAN NGỐ</t>
+  </si>
+  <si>
+    <t>SET ÁO LAYER BA LỖ PHỐI HAI DÂY TƠ BỒNG BỀNH</t>
+  </si>
+  <si>
+    <t>Áo Thun Nữ Cổ Thủy Thủ Phong Cách Hàn Quốc</t>
+  </si>
+  <si>
+    <t>ÁO CỔ YẾM BABYDOLL THÊU HOA</t>
+  </si>
+  <si>
+    <t>Áo Sát Nách Chấm Bi Cổ Sơ Mi Thắt Nơ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Set Áo Khoác Ren Móc Phối Áo Hai </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Quần Bí Nơ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chân Váy Vải Lông </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo thun nữ tay ngắn cổ trụ </t>
+  </si>
+  <si>
+    <t>CHÂN VÁY DÀI XẾP TẦNG</t>
+  </si>
+  <si>
+    <t>CHÂN VÁY REN TẦNG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Áo thun ngắn tay in hình </t>
   </si>
 </sst>
 </file>
@@ -6997,4 +7701,2376 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9001EBAE-A98A-4AAB-8066-D198D45A62E9}">
+  <dimension ref="A1:F102"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.44140625" customWidth="1"/>
+    <col min="2" max="2" width="56.88671875" customWidth="1"/>
+    <col min="3" max="3" width="46.5546875" customWidth="1"/>
+    <col min="4" max="4" width="44.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="19.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>608</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>684</v>
+      </c>
+      <c r="C3" t="s">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>686</v>
+      </c>
+      <c r="C4" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" t="s">
+        <v>688</v>
+      </c>
+      <c r="C5" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s">
+        <v>805</v>
+      </c>
+      <c r="C6" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>806</v>
+      </c>
+      <c r="C7" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
+        <v>807</v>
+      </c>
+      <c r="C8" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" t="s">
+        <v>808</v>
+      </c>
+      <c r="C9" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>809</v>
+      </c>
+      <c r="C10" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>810</v>
+      </c>
+      <c r="C11" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>811</v>
+      </c>
+      <c r="C12" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13" t="s">
+        <v>812</v>
+      </c>
+      <c r="C13" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" t="s">
+        <v>813</v>
+      </c>
+      <c r="C14" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>814</v>
+      </c>
+      <c r="C15" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>815</v>
+      </c>
+      <c r="C16" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>15</v>
+      </c>
+      <c r="B17" t="s">
+        <v>816</v>
+      </c>
+      <c r="C17" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" t="s">
+        <v>817</v>
+      </c>
+      <c r="C18" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>818</v>
+      </c>
+      <c r="C19" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" t="s">
+        <v>819</v>
+      </c>
+      <c r="C20" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <v>19</v>
+      </c>
+      <c r="B21" t="s">
+        <v>820</v>
+      </c>
+      <c r="C21" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>821</v>
+      </c>
+      <c r="C22" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23" t="s">
+        <v>822</v>
+      </c>
+      <c r="C23" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
+        <v>823</v>
+      </c>
+      <c r="C24" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25" t="s">
+        <v>824</v>
+      </c>
+      <c r="C25" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" t="s">
+        <v>825</v>
+      </c>
+      <c r="C26" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>826</v>
+      </c>
+      <c r="C27" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" t="s">
+        <v>827</v>
+      </c>
+      <c r="C28" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>27</v>
+      </c>
+      <c r="B29" t="s">
+        <v>828</v>
+      </c>
+      <c r="C29" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" t="s">
+        <v>829</v>
+      </c>
+      <c r="C30" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>830</v>
+      </c>
+      <c r="C31" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" t="s">
+        <v>831</v>
+      </c>
+      <c r="C32" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <v>31</v>
+      </c>
+      <c r="B33" t="s">
+        <v>832</v>
+      </c>
+      <c r="C33" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" t="s">
+        <v>833</v>
+      </c>
+      <c r="C34" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <v>33</v>
+      </c>
+      <c r="B35" t="s">
+        <v>834</v>
+      </c>
+      <c r="C35" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" t="s">
+        <v>835</v>
+      </c>
+      <c r="C36" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>35</v>
+      </c>
+      <c r="B37" t="s">
+        <v>836</v>
+      </c>
+      <c r="C37" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" t="s">
+        <v>837</v>
+      </c>
+      <c r="C38" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>37</v>
+      </c>
+      <c r="B39" t="s">
+        <v>838</v>
+      </c>
+      <c r="C39" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" t="s">
+        <v>839</v>
+      </c>
+      <c r="C40" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>39</v>
+      </c>
+      <c r="B41" t="s">
+        <v>840</v>
+      </c>
+      <c r="C41" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" t="s">
+        <v>726</v>
+      </c>
+      <c r="C42" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>728</v>
+      </c>
+      <c r="C43" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" t="s">
+        <v>730</v>
+      </c>
+      <c r="C44" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A45" s="3">
+        <v>43</v>
+      </c>
+      <c r="B45" t="s">
+        <v>732</v>
+      </c>
+      <c r="C45" t="s">
+        <v>733</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" t="s">
+        <v>734</v>
+      </c>
+      <c r="C46" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A47" s="3">
+        <v>45</v>
+      </c>
+      <c r="B47" t="s">
+        <v>736</v>
+      </c>
+      <c r="C47" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" t="s">
+        <v>738</v>
+      </c>
+      <c r="C48" t="s">
+        <v>739</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A49" s="3">
+        <v>47</v>
+      </c>
+      <c r="B49" t="s">
+        <v>740</v>
+      </c>
+      <c r="C49" t="s">
+        <v>741</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>742</v>
+      </c>
+      <c r="C50" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A51" s="3">
+        <v>49</v>
+      </c>
+      <c r="B51" t="s">
+        <v>744</v>
+      </c>
+      <c r="C51" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" t="s">
+        <v>746</v>
+      </c>
+      <c r="C52" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A53" s="3">
+        <v>51</v>
+      </c>
+      <c r="B53" t="s">
+        <v>748</v>
+      </c>
+      <c r="C53" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A54" s="3">
+        <v>52</v>
+      </c>
+      <c r="B54" t="s">
+        <v>750</v>
+      </c>
+      <c r="C54" t="s">
+        <v>751</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A55" s="3">
+        <v>53</v>
+      </c>
+      <c r="B55" t="s">
+        <v>752</v>
+      </c>
+      <c r="C55" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A56" s="3">
+        <v>54</v>
+      </c>
+      <c r="B56" t="s">
+        <v>754</v>
+      </c>
+      <c r="C56" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A57" s="3">
+        <v>55</v>
+      </c>
+      <c r="B57" t="s">
+        <v>756</v>
+      </c>
+      <c r="C57" t="s">
+        <v>757</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A58" s="3">
+        <v>56</v>
+      </c>
+      <c r="B58" t="s">
+        <v>758</v>
+      </c>
+      <c r="C58" t="s">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A59" s="3">
+        <v>57</v>
+      </c>
+      <c r="B59" t="s">
+        <v>760</v>
+      </c>
+      <c r="C59" t="s">
+        <v>761</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A60" s="3">
+        <v>58</v>
+      </c>
+      <c r="B60" t="s">
+        <v>762</v>
+      </c>
+      <c r="C60" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A61" s="3">
+        <v>59</v>
+      </c>
+      <c r="B61" t="s">
+        <v>764</v>
+      </c>
+      <c r="C61" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A62" s="3">
+        <v>60</v>
+      </c>
+      <c r="B62" t="s">
+        <v>766</v>
+      </c>
+      <c r="C62" t="s">
+        <v>767</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A63" s="3">
+        <v>61</v>
+      </c>
+      <c r="B63" t="s">
+        <v>768</v>
+      </c>
+      <c r="C63" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A64" s="3">
+        <v>62</v>
+      </c>
+      <c r="B64" t="s">
+        <v>770</v>
+      </c>
+      <c r="C64" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="3">
+        <v>63</v>
+      </c>
+      <c r="B65" t="s">
+        <v>772</v>
+      </c>
+      <c r="C65" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="3">
+        <v>64</v>
+      </c>
+      <c r="B66" t="s">
+        <v>774</v>
+      </c>
+      <c r="C66" t="s">
+        <v>775</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="3">
+        <v>65</v>
+      </c>
+      <c r="B67" t="s">
+        <v>776</v>
+      </c>
+      <c r="C67" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="3">
+        <v>66</v>
+      </c>
+      <c r="B68" t="s">
+        <v>778</v>
+      </c>
+      <c r="C68" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="3">
+        <v>67</v>
+      </c>
+      <c r="B69" t="s">
+        <v>780</v>
+      </c>
+      <c r="C69" t="s">
+        <v>781</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A70" s="3">
+        <v>68</v>
+      </c>
+      <c r="B70" t="s">
+        <v>782</v>
+      </c>
+      <c r="C70" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="3">
+        <v>69</v>
+      </c>
+      <c r="B71" t="s">
+        <v>784</v>
+      </c>
+      <c r="C71" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="3">
+        <v>70</v>
+      </c>
+      <c r="B72" t="s">
+        <v>786</v>
+      </c>
+      <c r="C72" t="s">
+        <v>787</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="3">
+        <v>71</v>
+      </c>
+      <c r="B73" t="s">
+        <v>788</v>
+      </c>
+      <c r="C73" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="3">
+        <v>72</v>
+      </c>
+      <c r="B74" t="s">
+        <v>790</v>
+      </c>
+      <c r="C74" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A75" s="3">
+        <v>73</v>
+      </c>
+      <c r="B75" t="s">
+        <v>792</v>
+      </c>
+      <c r="C75" t="s">
+        <v>793</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="3">
+        <v>74</v>
+      </c>
+      <c r="B76" t="s">
+        <v>794</v>
+      </c>
+      <c r="C76" t="s">
+        <v>795</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="3">
+        <v>75</v>
+      </c>
+      <c r="B77" t="s">
+        <v>796</v>
+      </c>
+      <c r="C77" t="s">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="3">
+        <v>76</v>
+      </c>
+      <c r="B78" t="s">
+        <v>798</v>
+      </c>
+      <c r="C78" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="3">
+        <v>77</v>
+      </c>
+      <c r="B79" t="s">
+        <v>800</v>
+      </c>
+      <c r="C79" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="3">
+        <v>78</v>
+      </c>
+      <c r="B80" t="s">
+        <v>802</v>
+      </c>
+      <c r="C80" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" s="3">
+        <v>79</v>
+      </c>
+      <c r="B81" t="s">
+        <v>841</v>
+      </c>
+      <c r="C81" t="s">
+        <v>804</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" s="3">
+        <v>80</v>
+      </c>
+      <c r="B82" s="19"/>
+      <c r="C82" s="14"/>
+      <c r="D82" s="14"/>
+      <c r="E82" s="14"/>
+      <c r="F82" s="1"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" s="3">
+        <v>81</v>
+      </c>
+      <c r="B83" s="19"/>
+      <c r="C83" s="14"/>
+      <c r="D83" s="14"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="1"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" s="3">
+        <v>82</v>
+      </c>
+      <c r="B84" s="19"/>
+      <c r="C84" s="9"/>
+      <c r="D84" s="9"/>
+      <c r="E84" s="9"/>
+      <c r="F84" s="1"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" s="3">
+        <v>83</v>
+      </c>
+      <c r="B85" s="19"/>
+      <c r="C85" s="14"/>
+      <c r="D85" s="14"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="1"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" s="3">
+        <v>84</v>
+      </c>
+      <c r="B86" s="19"/>
+      <c r="C86" s="14"/>
+      <c r="D86" s="14"/>
+      <c r="E86" s="14"/>
+      <c r="F86" s="1"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" s="3">
+        <v>85</v>
+      </c>
+      <c r="B87" s="19"/>
+      <c r="C87" s="14"/>
+      <c r="D87" s="14"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="1"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" s="3">
+        <v>86</v>
+      </c>
+      <c r="B88" s="19"/>
+      <c r="C88" s="14"/>
+      <c r="D88" s="14"/>
+      <c r="E88" s="14"/>
+      <c r="F88" s="1"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" s="3">
+        <v>87</v>
+      </c>
+      <c r="B89" s="19"/>
+      <c r="C89" s="14"/>
+      <c r="D89" s="14"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="1"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" s="3">
+        <v>88</v>
+      </c>
+      <c r="B90" s="19"/>
+      <c r="C90" s="14"/>
+      <c r="D90" s="14"/>
+      <c r="E90" s="14"/>
+      <c r="F90" s="1"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" s="3">
+        <v>89</v>
+      </c>
+      <c r="B91" s="19"/>
+      <c r="C91" s="14"/>
+      <c r="D91" s="14"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="1"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" s="3">
+        <v>90</v>
+      </c>
+      <c r="B92" s="19"/>
+      <c r="C92" s="14"/>
+      <c r="D92" s="14"/>
+      <c r="E92" s="14"/>
+      <c r="F92" s="1"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="3">
+        <v>91</v>
+      </c>
+      <c r="B93" s="19"/>
+      <c r="C93" s="14"/>
+      <c r="D93" s="14"/>
+      <c r="E93" s="14"/>
+      <c r="F93" s="1"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" s="3">
+        <v>92</v>
+      </c>
+      <c r="B94" s="19"/>
+      <c r="C94" s="14"/>
+      <c r="D94" s="14"/>
+      <c r="E94" s="14"/>
+      <c r="F94" s="1"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" s="3">
+        <v>93</v>
+      </c>
+      <c r="B95" s="19"/>
+      <c r="C95" s="14"/>
+      <c r="D95" s="14"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="1"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" s="3">
+        <v>94</v>
+      </c>
+      <c r="B96" s="19"/>
+      <c r="C96" s="14"/>
+      <c r="D96" s="14"/>
+      <c r="E96" s="14"/>
+      <c r="F96" s="1"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" s="3">
+        <v>95</v>
+      </c>
+      <c r="B97" s="19"/>
+      <c r="C97" s="14"/>
+      <c r="D97" s="14"/>
+      <c r="E97" s="14"/>
+      <c r="F97" s="1"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="3">
+        <v>96</v>
+      </c>
+      <c r="B98" s="19"/>
+      <c r="C98" s="14"/>
+      <c r="D98" s="14"/>
+      <c r="E98" s="14"/>
+      <c r="F98" s="1"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="3">
+        <v>97</v>
+      </c>
+      <c r="B99" s="19"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="14"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="1"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="3">
+        <v>98</v>
+      </c>
+      <c r="B100" s="19"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="14"/>
+      <c r="E100" s="14"/>
+      <c r="F100" s="1"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="3">
+        <v>99</v>
+      </c>
+      <c r="B101" s="19"/>
+      <c r="C101" s="14"/>
+      <c r="D101" s="14"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="1"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="3">
+        <v>100</v>
+      </c>
+      <c r="B102" s="19"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="14"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B1D917C-F7D3-42CF-8398-0DC6E7E7A328}">
+  <dimension ref="A1:F102"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="6.21875" customWidth="1"/>
+    <col min="2" max="3" width="36.5546875" customWidth="1"/>
+    <col min="4" max="4" width="37.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" ht="19.2" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>608</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>610</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>605</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="C3" s="17" t="s">
+        <v>611</v>
+      </c>
+      <c r="D3" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E3" s="17"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>613</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="E4" s="5"/>
+      <c r="F4" s="6"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>616</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>618</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>617</v>
+      </c>
+      <c r="E5" s="5"/>
+      <c r="F5" s="6"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>620</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>621</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="6"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>622</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>623</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>624</v>
+      </c>
+      <c r="E7" s="5"/>
+      <c r="F7" s="6"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>626</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>625</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>627</v>
+      </c>
+      <c r="E8" s="5"/>
+      <c r="F8" s="6"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>629</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>628</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>630</v>
+      </c>
+      <c r="E9" s="5"/>
+      <c r="F9" s="6"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>631</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>632</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="E10" s="5"/>
+      <c r="F10" s="6"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>635</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>633</v>
+      </c>
+      <c r="E11" s="5"/>
+      <c r="F11" s="6"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>637</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>636</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>638</v>
+      </c>
+      <c r="E12" s="5"/>
+      <c r="F12" s="6"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>639</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="E13" s="5"/>
+      <c r="F13" s="6"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7" t="s">
+        <v>642</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>643</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>644</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>645</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>646</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>647</v>
+      </c>
+      <c r="E15" s="10"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>648</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>649</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>644</v>
+      </c>
+      <c r="E16" s="10"/>
+      <c r="F16" s="6"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A17" s="3">
+        <v>15</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>650</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>651</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>652</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="6"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>653</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>654</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>633</v>
+      </c>
+      <c r="E18" s="10"/>
+      <c r="F18" s="6"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A19" s="3">
+        <v>17</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>655</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>656</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>647</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="6"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>657</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>658</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>659</v>
+      </c>
+      <c r="E20" s="10"/>
+      <c r="F20" s="6"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A21" s="3">
+        <v>19</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>660</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>662</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>661</v>
+      </c>
+      <c r="E21" s="10"/>
+      <c r="F21" s="6"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>663</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>664</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>661</v>
+      </c>
+      <c r="E22" s="10"/>
+      <c r="F22" s="6"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>665</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>666</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>667</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="6"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>668</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>669</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>670</v>
+      </c>
+      <c r="E24" s="10"/>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>671</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>672</v>
+      </c>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="6"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>673</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>674</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>675</v>
+      </c>
+      <c r="E26" s="10"/>
+      <c r="F26" s="6"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>676</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>677</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>667</v>
+      </c>
+      <c r="E27" s="10"/>
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>679</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>641</v>
+      </c>
+      <c r="E28" s="10"/>
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A29" s="3">
+        <v>27</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>680</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>681</v>
+      </c>
+      <c r="D29" s="10" t="s">
+        <v>670</v>
+      </c>
+      <c r="E29" s="10"/>
+      <c r="F29" s="6"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>682</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>683</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>670</v>
+      </c>
+      <c r="E30" s="10"/>
+      <c r="F30" s="6"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A31" s="3">
+        <v>29</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="10"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="10"/>
+      <c r="F31" s="6"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="6"/>
+      <c r="C32" s="10"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="10"/>
+      <c r="F32" s="6"/>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A33" s="3">
+        <v>31</v>
+      </c>
+      <c r="B33" s="7"/>
+      <c r="C33" s="10"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="6"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" s="7"/>
+      <c r="C34" s="10"/>
+      <c r="D34" s="10"/>
+      <c r="E34" s="10"/>
+      <c r="F34" s="6"/>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A35" s="3">
+        <v>33</v>
+      </c>
+      <c r="B35" s="7"/>
+      <c r="C35" s="10"/>
+      <c r="D35" s="10"/>
+      <c r="E35" s="10"/>
+      <c r="F35" s="6"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" s="7"/>
+      <c r="C36" s="10"/>
+      <c r="D36" s="10"/>
+      <c r="E36" s="10"/>
+      <c r="F36" s="6"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A37" s="3">
+        <v>35</v>
+      </c>
+      <c r="B37" s="7"/>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="6"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="7"/>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="10"/>
+      <c r="F38" s="6"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A39" s="3">
+        <v>37</v>
+      </c>
+      <c r="B39" s="7"/>
+      <c r="C39" s="10"/>
+      <c r="D39" s="10"/>
+      <c r="E39" s="10"/>
+      <c r="F39" s="6"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="7"/>
+      <c r="C40" s="10"/>
+      <c r="D40" s="10"/>
+      <c r="E40" s="10"/>
+      <c r="F40" s="6"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A41" s="3">
+        <v>39</v>
+      </c>
+      <c r="B41" s="18"/>
+      <c r="C41" s="10"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="6"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" s="7"/>
+      <c r="C42" s="10"/>
+      <c r="D42" s="10"/>
+      <c r="E42" s="10"/>
+      <c r="F42" s="6"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A43" s="3">
+        <v>41</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="10"/>
+      <c r="D43" s="10"/>
+      <c r="E43" s="10"/>
+      <c r="F43" s="6"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" s="7"/>
+      <c r="C44" s="10"/>
+      <c r="D44" s="10"/>
+      <c r="E44" s="10"/>
+      <c r="F44" s="6"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A45" s="3">
+        <v>43</v>
+      </c>
+      <c r="B45" s="7"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
+      <c r="E45" s="10"/>
+      <c r="F45" s="6"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="7"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="6"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A47" s="3">
+        <v>45</v>
+      </c>
+      <c r="B47" s="7"/>
+      <c r="C47" s="10"/>
+      <c r="D47" s="10"/>
+      <c r="E47" s="10"/>
+      <c r="F47" s="6"/>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" s="7"/>
+      <c r="C48" s="10"/>
+      <c r="D48" s="10"/>
+      <c r="E48" s="10"/>
+      <c r="F48" s="6"/>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A49" s="3">
+        <v>47</v>
+      </c>
+      <c r="B49" s="7"/>
+      <c r="C49" s="10"/>
+      <c r="D49" s="10"/>
+      <c r="E49" s="10"/>
+      <c r="F49" s="6"/>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" s="7"/>
+      <c r="C50" s="10"/>
+      <c r="D50" s="10"/>
+      <c r="E50" s="10"/>
+      <c r="F50" s="6"/>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A51" s="3">
+        <v>49</v>
+      </c>
+      <c r="B51" s="7"/>
+      <c r="C51" s="10"/>
+      <c r="D51" s="10"/>
+      <c r="E51" s="10"/>
+      <c r="F51" s="6"/>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" s="7"/>
+      <c r="C52" s="10"/>
+      <c r="D52" s="10"/>
+      <c r="E52" s="10"/>
+      <c r="F52" s="6"/>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A53" s="3">
+        <v>51</v>
+      </c>
+      <c r="B53" s="7"/>
+      <c r="C53" s="10"/>
+      <c r="D53" s="10"/>
+      <c r="E53" s="10"/>
+      <c r="F53" s="6"/>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A54" s="3">
+        <v>52</v>
+      </c>
+      <c r="B54" s="7"/>
+      <c r="C54" s="10"/>
+      <c r="D54" s="10"/>
+      <c r="E54" s="10"/>
+      <c r="F54" s="6"/>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A55" s="3">
+        <v>53</v>
+      </c>
+      <c r="B55" s="7"/>
+      <c r="C55" s="10"/>
+      <c r="D55" s="10"/>
+      <c r="E55" s="10"/>
+      <c r="F55" s="6"/>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A56" s="3">
+        <v>54</v>
+      </c>
+      <c r="B56" s="7"/>
+      <c r="C56" s="10"/>
+      <c r="D56" s="10"/>
+      <c r="E56" s="10"/>
+      <c r="F56" s="6"/>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A57" s="3">
+        <v>55</v>
+      </c>
+      <c r="B57" s="7"/>
+      <c r="C57" s="5"/>
+      <c r="D57" s="5"/>
+      <c r="E57" s="5"/>
+      <c r="F57" s="7"/>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A58" s="3">
+        <v>56</v>
+      </c>
+      <c r="B58" s="7"/>
+      <c r="C58" s="5"/>
+      <c r="D58" s="5"/>
+      <c r="E58" s="5"/>
+      <c r="F58" s="7"/>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A59" s="3">
+        <v>57</v>
+      </c>
+      <c r="B59" s="7"/>
+      <c r="C59" s="5"/>
+      <c r="D59" s="5"/>
+      <c r="E59" s="5"/>
+      <c r="F59" s="7"/>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A60" s="3">
+        <v>58</v>
+      </c>
+      <c r="B60" s="7"/>
+      <c r="C60" s="5"/>
+      <c r="D60" s="5"/>
+      <c r="E60" s="5"/>
+      <c r="F60" s="7"/>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A61" s="3">
+        <v>59</v>
+      </c>
+      <c r="B61" s="7"/>
+      <c r="C61" s="5"/>
+      <c r="D61" s="5"/>
+      <c r="E61" s="5"/>
+      <c r="F61" s="7"/>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A62" s="3">
+        <v>60</v>
+      </c>
+      <c r="B62" s="7"/>
+      <c r="C62" s="5"/>
+      <c r="D62" s="5"/>
+      <c r="E62" s="5"/>
+      <c r="F62" s="7"/>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A63" s="3">
+        <v>61</v>
+      </c>
+      <c r="B63" s="7"/>
+      <c r="C63" s="5"/>
+      <c r="D63" s="5"/>
+      <c r="E63" s="5"/>
+      <c r="F63" s="7"/>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A64" s="3">
+        <v>62</v>
+      </c>
+      <c r="B64" s="7"/>
+      <c r="C64" s="5"/>
+      <c r="D64" s="5"/>
+      <c r="E64" s="5"/>
+      <c r="F64" s="7"/>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A65" s="3">
+        <v>63</v>
+      </c>
+      <c r="B65" s="7"/>
+      <c r="C65" s="5"/>
+      <c r="D65" s="5"/>
+      <c r="E65" s="5"/>
+      <c r="F65" s="7"/>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="3">
+        <v>64</v>
+      </c>
+      <c r="B66" s="7"/>
+      <c r="C66" s="5"/>
+      <c r="D66" s="5"/>
+      <c r="E66" s="5"/>
+      <c r="F66" s="7"/>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="3">
+        <v>65</v>
+      </c>
+      <c r="B67" s="7"/>
+      <c r="C67" s="5"/>
+      <c r="D67" s="5"/>
+      <c r="E67" s="5"/>
+      <c r="F67" s="7"/>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="3">
+        <v>66</v>
+      </c>
+      <c r="B68" s="7"/>
+      <c r="C68" s="5"/>
+      <c r="D68" s="5"/>
+      <c r="E68" s="5"/>
+      <c r="F68" s="7"/>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="3">
+        <v>67</v>
+      </c>
+      <c r="B69" s="7"/>
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+      <c r="F69" s="7"/>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="3">
+        <v>68</v>
+      </c>
+      <c r="B70" s="7"/>
+      <c r="C70" s="5"/>
+      <c r="D70" s="5"/>
+      <c r="E70" s="5"/>
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="3">
+        <v>69</v>
+      </c>
+      <c r="B71" s="7"/>
+      <c r="C71" s="5"/>
+      <c r="D71" s="5"/>
+      <c r="E71" s="5"/>
+      <c r="F71" s="7"/>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="3">
+        <v>70</v>
+      </c>
+      <c r="B72" s="7"/>
+      <c r="C72" s="5"/>
+      <c r="D72" s="5"/>
+      <c r="E72" s="5"/>
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="3">
+        <v>71</v>
+      </c>
+      <c r="B73" s="19"/>
+      <c r="C73" s="14"/>
+      <c r="D73" s="14"/>
+      <c r="E73" s="14"/>
+      <c r="F73" s="1"/>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="3">
+        <v>72</v>
+      </c>
+      <c r="B74" s="19"/>
+      <c r="C74" s="14"/>
+      <c r="D74" s="14"/>
+      <c r="E74" s="14"/>
+      <c r="F74" s="1"/>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="3">
+        <v>73</v>
+      </c>
+      <c r="B75" s="19"/>
+      <c r="C75" s="14"/>
+      <c r="D75" s="14"/>
+      <c r="E75" s="14"/>
+      <c r="F75" s="1"/>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A76" s="3">
+        <v>74</v>
+      </c>
+      <c r="B76" s="19"/>
+      <c r="C76" s="14"/>
+      <c r="D76" s="14"/>
+      <c r="E76" s="14"/>
+      <c r="F76" s="1"/>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="3">
+        <v>75</v>
+      </c>
+      <c r="B77" s="19"/>
+      <c r="C77" s="14"/>
+      <c r="D77" s="14"/>
+      <c r="E77" s="14"/>
+      <c r="F77" s="1"/>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="3">
+        <v>76</v>
+      </c>
+      <c r="B78" s="19"/>
+      <c r="C78" s="14"/>
+      <c r="D78" s="14"/>
+      <c r="E78" s="14"/>
+      <c r="F78" s="1"/>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A79" s="3">
+        <v>77</v>
+      </c>
+      <c r="B79" s="19"/>
+      <c r="C79" s="14"/>
+      <c r="D79" s="14"/>
+      <c r="E79" s="14"/>
+      <c r="F79" s="1"/>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A80" s="3">
+        <v>78</v>
+      </c>
+      <c r="B80" s="19"/>
+      <c r="C80" s="14"/>
+      <c r="D80" s="14"/>
+      <c r="E80" s="14"/>
+      <c r="F80" s="1"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A81" s="3">
+        <v>79</v>
+      </c>
+      <c r="B81" s="19"/>
+      <c r="C81" s="14"/>
+      <c r="D81" s="14"/>
+      <c r="E81" s="14"/>
+      <c r="F81" s="1"/>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A82" s="3">
+        <v>80</v>
+      </c>
+      <c r="B82" s="19"/>
+      <c r="C82" s="14"/>
+      <c r="D82" s="14"/>
+      <c r="E82" s="14"/>
+      <c r="F82" s="1"/>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A83" s="3">
+        <v>81</v>
+      </c>
+      <c r="B83" s="19"/>
+      <c r="C83" s="14"/>
+      <c r="D83" s="14"/>
+      <c r="E83" s="14"/>
+      <c r="F83" s="1"/>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A84" s="3">
+        <v>82</v>
+      </c>
+      <c r="B84" s="19"/>
+      <c r="C84" s="9"/>
+      <c r="D84" s="9"/>
+      <c r="E84" s="9"/>
+      <c r="F84" s="1"/>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A85" s="3">
+        <v>83</v>
+      </c>
+      <c r="B85" s="19"/>
+      <c r="C85" s="14"/>
+      <c r="D85" s="14"/>
+      <c r="E85" s="14"/>
+      <c r="F85" s="1"/>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A86" s="3">
+        <v>84</v>
+      </c>
+      <c r="B86" s="19"/>
+      <c r="C86" s="14"/>
+      <c r="D86" s="14"/>
+      <c r="E86" s="14"/>
+      <c r="F86" s="1"/>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A87" s="3">
+        <v>85</v>
+      </c>
+      <c r="B87" s="19"/>
+      <c r="C87" s="14"/>
+      <c r="D87" s="14"/>
+      <c r="E87" s="14"/>
+      <c r="F87" s="1"/>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A88" s="3">
+        <v>86</v>
+      </c>
+      <c r="B88" s="19"/>
+      <c r="C88" s="14"/>
+      <c r="D88" s="14"/>
+      <c r="E88" s="14"/>
+      <c r="F88" s="1"/>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A89" s="3">
+        <v>87</v>
+      </c>
+      <c r="B89" s="19"/>
+      <c r="C89" s="14"/>
+      <c r="D89" s="14"/>
+      <c r="E89" s="14"/>
+      <c r="F89" s="1"/>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A90" s="3">
+        <v>88</v>
+      </c>
+      <c r="B90" s="19"/>
+      <c r="C90" s="14"/>
+      <c r="D90" s="14"/>
+      <c r="E90" s="14"/>
+      <c r="F90" s="1"/>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A91" s="3">
+        <v>89</v>
+      </c>
+      <c r="B91" s="19"/>
+      <c r="C91" s="14"/>
+      <c r="D91" s="14"/>
+      <c r="E91" s="14"/>
+      <c r="F91" s="1"/>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" s="3">
+        <v>90</v>
+      </c>
+      <c r="B92" s="19"/>
+      <c r="C92" s="14"/>
+      <c r="D92" s="14"/>
+      <c r="E92" s="14"/>
+      <c r="F92" s="1"/>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="3">
+        <v>91</v>
+      </c>
+      <c r="B93" s="19"/>
+      <c r="C93" s="14"/>
+      <c r="D93" s="14"/>
+      <c r="E93" s="14"/>
+      <c r="F93" s="1"/>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A94" s="3">
+        <v>92</v>
+      </c>
+      <c r="B94" s="19"/>
+      <c r="C94" s="14"/>
+      <c r="D94" s="14"/>
+      <c r="E94" s="14"/>
+      <c r="F94" s="1"/>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" s="3">
+        <v>93</v>
+      </c>
+      <c r="B95" s="19"/>
+      <c r="C95" s="14"/>
+      <c r="D95" s="14"/>
+      <c r="E95" s="14"/>
+      <c r="F95" s="1"/>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A96" s="3">
+        <v>94</v>
+      </c>
+      <c r="B96" s="19"/>
+      <c r="C96" s="14"/>
+      <c r="D96" s="14"/>
+      <c r="E96" s="14"/>
+      <c r="F96" s="1"/>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" s="3">
+        <v>95</v>
+      </c>
+      <c r="B97" s="19"/>
+      <c r="C97" s="14"/>
+      <c r="D97" s="14"/>
+      <c r="E97" s="14"/>
+      <c r="F97" s="1"/>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="3">
+        <v>96</v>
+      </c>
+      <c r="B98" s="19"/>
+      <c r="C98" s="14"/>
+      <c r="D98" s="14"/>
+      <c r="E98" s="14"/>
+      <c r="F98" s="1"/>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="3">
+        <v>97</v>
+      </c>
+      <c r="B99" s="19"/>
+      <c r="C99" s="14"/>
+      <c r="D99" s="14"/>
+      <c r="E99" s="14"/>
+      <c r="F99" s="1"/>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="3">
+        <v>98</v>
+      </c>
+      <c r="B100" s="19"/>
+      <c r="C100" s="14"/>
+      <c r="D100" s="14"/>
+      <c r="E100" s="14"/>
+      <c r="F100" s="1"/>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="3">
+        <v>99</v>
+      </c>
+      <c r="B101" s="19"/>
+      <c r="C101" s="14"/>
+      <c r="D101" s="14"/>
+      <c r="E101" s="14"/>
+      <c r="F101" s="1"/>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="3">
+        <v>100</v>
+      </c>
+      <c r="B102" s="19"/>
+      <c r="C102" s="14"/>
+      <c r="D102" s="14"/>
+      <c r="E102" s="14"/>
+      <c r="F102" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="C3" r:id="rId1" xr:uid="{FB450A53-B758-4466-B275-DBC75078C58D}"/>
+    <hyperlink ref="C4" r:id="rId2" xr:uid="{94CCE20D-0ABA-40B2-A7F6-0F1030FCA65D}"/>
+    <hyperlink ref="C5" r:id="rId3" xr:uid="{E8966332-3F84-4197-A830-7B05D800E0D0}"/>
+    <hyperlink ref="C6" r:id="rId4" xr:uid="{3CF770CB-54EC-4016-9BC9-B1C1631B6EC4}"/>
+    <hyperlink ref="C7" r:id="rId5" xr:uid="{0A084092-C88B-4C90-B89A-F838E59B1DA4}"/>
+    <hyperlink ref="C8" r:id="rId6" xr:uid="{FAEA679A-BB95-4AD0-A386-4AC037E26C28}"/>
+    <hyperlink ref="C9" r:id="rId7" xr:uid="{FC377E94-6C2E-4BEB-B859-3FB15B08F31C}"/>
+    <hyperlink ref="C10" r:id="rId8" xr:uid="{577093F6-AFEF-445F-927D-E484CF26FCFB}"/>
+    <hyperlink ref="C11" r:id="rId9" xr:uid="{5D6125D4-C91A-49B2-A19A-44EADA018743}"/>
+    <hyperlink ref="C12" r:id="rId10" xr:uid="{49E64C35-C668-467B-B6C0-F972DA338473}"/>
+    <hyperlink ref="C13" r:id="rId11" xr:uid="{C8AABAE1-1188-4621-B2CC-8DF4F5F43A54}"/>
+    <hyperlink ref="C14" r:id="rId12" xr:uid="{1F962A3E-48F7-492F-9014-1BCBD5776A5A}"/>
+    <hyperlink ref="C15" r:id="rId13" xr:uid="{6786B77F-4703-4392-B6A6-33F6C9E01492}"/>
+    <hyperlink ref="C16" r:id="rId14" xr:uid="{854DF863-F732-47C4-BD8B-100EDBBFBCBD}"/>
+    <hyperlink ref="C17" r:id="rId15" xr:uid="{B7EB6A76-178E-4EDC-960B-9BAC51C1A55E}"/>
+    <hyperlink ref="C18" r:id="rId16" xr:uid="{E96193F9-2FC2-4768-AD9D-2A87E6B284BB}"/>
+    <hyperlink ref="C19" r:id="rId17" xr:uid="{DBA98719-CADF-4177-A21E-73D90F9E09F4}"/>
+    <hyperlink ref="C20" r:id="rId18" xr:uid="{FB4E0039-E979-4508-8AF5-3A64858388AB}"/>
+    <hyperlink ref="C21" r:id="rId19" xr:uid="{76DD4345-85CE-4880-997A-D32EDBDE081A}"/>
+    <hyperlink ref="C22" r:id="rId20" xr:uid="{2A5F4480-2B86-4758-8EF7-557EDAD9DFB4}"/>
+    <hyperlink ref="C23" r:id="rId21" xr:uid="{B9013DE1-4E84-4BF0-97A8-EDFEE152CD53}"/>
+    <hyperlink ref="C24" r:id="rId22" xr:uid="{04350732-9F6C-4E10-B162-591C6C7CBBB5}"/>
+    <hyperlink ref="C25" r:id="rId23" xr:uid="{59682EEF-5353-45F7-B173-6397B3ADE4A8}"/>
+    <hyperlink ref="C26" r:id="rId24" xr:uid="{570CF8A9-4072-46D5-8DBA-A18C292D6A83}"/>
+    <hyperlink ref="C27" r:id="rId25" xr:uid="{87AED2AB-0AB5-4F9A-8EC3-EDA97D2D8731}"/>
+    <hyperlink ref="C28" r:id="rId26" xr:uid="{6F4453FF-A4EE-4168-B201-7FA06F1F735B}"/>
+    <hyperlink ref="C29" r:id="rId27" xr:uid="{17B064C0-5BC4-441F-9BC9-F5BEBBBDE6D4}"/>
+    <hyperlink ref="C30" r:id="rId28" xr:uid="{6F46CAE8-0D55-4AC1-AF33-4B9D08E8CBDB}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>